<commit_message>
Restrict LT contact set to operation_35_lt only
Drop the two operation_35_lt_nick carve-ins added in the previous commit
(Jen Hensley, Sophia Schneider). The Nick list is captured elsewhere, so this
file is now a pure tag cut: operation_35_lt and nothing else.

80 contacts. Raters are Joanna Patterson (50), David Yang (30) and Victoria
Mayo (1 co-rater). 15 fit the size+geo criteria, matching the tag-level count
computed independently against the database.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vpqx8vJoRPj3j5ZpESJHvv
</commit_message>
<xml_diff>
--- a/Operation35_LT_Contacts.xlsx
+++ b/Operation35_LT_Contacts.xlsx
@@ -11,7 +11,7 @@
     <sheet name="READ ME" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LT x Fit'!$A$1:$U$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LT x Fit'!$A$1:$U$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U83"/>
+  <dimension ref="A1:U81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1859,22 +1859,22 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Uniswap Labs</t>
+          <t>Urban Upbound (formerly ERDA)</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Sophia Schneider</t>
+          <t>Bishop Mitchell G. Taylor</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Events</t>
+          <t>Co-Founder &amp; Ceo</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Nonprofit</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1893,15 +1893,19 @@
         </is>
       </c>
       <c r="K16" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>Joanna Patterson | Stefano Barros | Victoria Mayo</t>
+          <t>David Yang</t>
         </is>
       </c>
       <c r="M16" s="4" t="inlineStr"/>
-      <c r="N16" s="4" t="inlineStr"/>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/bishop-mitchell-g-taylor-994715a</t>
+        </is>
+      </c>
       <c r="O16" s="5" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr">
         <is>
@@ -1911,101 +1915,97 @@
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="n">
-        <v>12434</v>
+        <v>2893</v>
       </c>
       <c r="T16" s="4" t="inlineStr">
         <is>
-          <t>10279</t>
+          <t>10311</t>
         </is>
       </c>
       <c r="U16" s="4" t="inlineStr">
         <is>
-          <t>LT_Nick list, but rated only by Joanna/Dave</t>
+          <t>Operation 35 — LT (Joanna / Dave)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Unknown — company not enriched</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Barrel Holdings</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Peter Kang</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Co-founder &amp; Chairman</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>1-10</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr"/>
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Urban Upbound (formerly ERDA)</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>Bishop Mitchell G. Taylor</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Co-Founder &amp; Ceo</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>Nonprofit</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>51-200</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>New York, NY</t>
-        </is>
-      </c>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L17" s="5" t="inlineStr">
+      <c r="K17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" s="7" t="inlineStr">
         <is>
           <t>David Yang</t>
         </is>
       </c>
-      <c r="M17" s="4" t="inlineStr"/>
-      <c r="N17" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/bishop-mitchell-g-taylor-994715a</t>
-        </is>
-      </c>
-      <c r="O17" s="5" t="inlineStr"/>
-      <c r="P17" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="Q17" s="4" t="inlineStr"/>
-      <c r="R17" s="4" t="inlineStr"/>
-      <c r="S17" s="4" t="n">
-        <v>2893</v>
-      </c>
-      <c r="T17" s="4" t="inlineStr">
-        <is>
-          <t>10311</t>
-        </is>
-      </c>
-      <c r="U17" s="4" t="inlineStr">
+      <c r="M17" s="6" t="inlineStr"/>
+      <c r="N17" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/peterkang34</t>
+        </is>
+      </c>
+      <c r="O17" s="7" t="inlineStr"/>
+      <c r="P17" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="Q17" s="6" t="inlineStr"/>
+      <c r="R17" s="6" t="inlineStr"/>
+      <c r="S17" s="6" t="n">
+        <v>6821</v>
+      </c>
+      <c r="T17" s="6" t="inlineStr">
+        <is>
+          <t>3122</t>
+        </is>
+      </c>
+      <c r="U17" s="6" t="inlineStr">
         <is>
           <t>Operation 35 — LT (Joanna / Dave)</t>
         </is>
@@ -2029,29 +2029,21 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>Barrel Holdings</t>
+          <t>Charney Companies LLC</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Peter Kang</t>
+          <t>Sam Charney</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Co-founder &amp; Chairman</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr">
-        <is>
-          <t>1-10</t>
-        </is>
-      </c>
+          <t>Founder and Principal</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr"/>
+      <c r="H18" s="6" t="inlineStr"/>
       <c r="I18" s="6" t="inlineStr"/>
       <c r="J18" s="6" t="inlineStr">
         <is>
@@ -2066,12 +2058,12 @@
           <t>David Yang</t>
         </is>
       </c>
-      <c r="M18" s="6" t="inlineStr"/>
-      <c r="N18" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/peterkang34</t>
-        </is>
-      </c>
+      <c r="M18" s="6" t="inlineStr">
+        <is>
+          <t>sam@charneycompanies.com</t>
+        </is>
+      </c>
+      <c r="N18" s="6" t="inlineStr"/>
       <c r="O18" s="7" t="inlineStr"/>
       <c r="P18" s="6" t="inlineStr">
         <is>
@@ -2081,11 +2073,11 @@
       <c r="Q18" s="6" t="inlineStr"/>
       <c r="R18" s="6" t="inlineStr"/>
       <c r="S18" s="6" t="n">
-        <v>6821</v>
+        <v>15047</v>
       </c>
       <c r="T18" s="6" t="inlineStr">
         <is>
-          <t>3122</t>
+          <t>11907</t>
         </is>
       </c>
       <c r="U18" s="6" t="inlineStr">
@@ -2112,21 +2104,29 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Charney Companies LLC</t>
+          <t>Crafted Action</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Sam Charney</t>
+          <t>Brad Baer</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>Founder and Principal</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr"/>
-      <c r="H19" s="6" t="inlineStr"/>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>1-10</t>
+        </is>
+      </c>
       <c r="I19" s="6" t="inlineStr"/>
       <c r="J19" s="6" t="inlineStr">
         <is>
@@ -2141,12 +2141,12 @@
           <t>David Yang</t>
         </is>
       </c>
-      <c r="M19" s="6" t="inlineStr">
-        <is>
-          <t>sam@charneycompanies.com</t>
-        </is>
-      </c>
-      <c r="N19" s="6" t="inlineStr"/>
+      <c r="M19" s="6" t="inlineStr"/>
+      <c r="N19" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/bbaer</t>
+        </is>
+      </c>
       <c r="O19" s="7" t="inlineStr"/>
       <c r="P19" s="6" t="inlineStr">
         <is>
@@ -2156,11 +2156,11 @@
       <c r="Q19" s="6" t="inlineStr"/>
       <c r="R19" s="6" t="inlineStr"/>
       <c r="S19" s="6" t="n">
-        <v>15047</v>
+        <v>6629</v>
       </c>
       <c r="T19" s="6" t="inlineStr">
         <is>
-          <t>11907</t>
+          <t>3965</t>
         </is>
       </c>
       <c r="U19" s="6" t="inlineStr">
@@ -2187,27 +2187,27 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Crafted Action</t>
+          <t>Prima Mode</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Brad Baer</t>
+          <t>Sei-Wook Kim</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>Founder &amp; CEO</t>
+          <t>Co-founder</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>1-10</t>
+          <t>51-200</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr"/>
@@ -2227,7 +2227,7 @@
       <c r="M20" s="6" t="inlineStr"/>
       <c r="N20" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/bbaer</t>
+          <t>https://www.linkedin.com/in/seiwookkim</t>
         </is>
       </c>
       <c r="O20" s="7" t="inlineStr"/>
@@ -2239,11 +2239,11 @@
       <c r="Q20" s="6" t="inlineStr"/>
       <c r="R20" s="6" t="inlineStr"/>
       <c r="S20" s="6" t="n">
-        <v>6629</v>
+        <v>6762</v>
       </c>
       <c r="T20" s="6" t="inlineStr">
         <is>
-          <t>3965</t>
+          <t>8045</t>
         </is>
       </c>
       <c r="U20" s="6" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Unassigned</t>
+          <t>David</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -2270,29 +2270,21 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Prima Mode</t>
+          <t>Puzzmo</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Sei-Wook Kim</t>
+          <t>Orta Therox</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>Co-founder</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>Retail</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>51-200</t>
-        </is>
-      </c>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr"/>
+      <c r="H21" s="6" t="inlineStr"/>
       <c r="I21" s="6" t="inlineStr"/>
       <c r="J21" s="6" t="inlineStr">
         <is>
@@ -2310,7 +2302,7 @@
       <c r="M21" s="6" t="inlineStr"/>
       <c r="N21" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/seiwookkim</t>
+          <t>https://www.linkedin.com/in/ortatherox/</t>
         </is>
       </c>
       <c r="O21" s="7" t="inlineStr"/>
@@ -2320,13 +2312,17 @@
         </is>
       </c>
       <c r="Q21" s="6" t="inlineStr"/>
-      <c r="R21" s="6" t="inlineStr"/>
+      <c r="R21" s="6" t="inlineStr">
+        <is>
+          <t>david@pursuit.org</t>
+        </is>
+      </c>
       <c r="S21" s="6" t="n">
-        <v>6762</v>
+        <v>14837</v>
       </c>
       <c r="T21" s="6" t="inlineStr">
         <is>
-          <t>8045</t>
+          <t>12535</t>
         </is>
       </c>
       <c r="U21" s="6" t="inlineStr">
@@ -2343,7 +2339,7 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>David</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -2353,21 +2349,29 @@
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Puzzmo</t>
+          <t>SHAY CPA P.C.</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Orta Therox</t>
+          <t>Akshay Shrimanker</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Co-Founder</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr"/>
-      <c r="H22" s="6" t="inlineStr"/>
+          <t>Chief Executive Officer</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>1-10</t>
+        </is>
+      </c>
       <c r="I22" s="6" t="inlineStr"/>
       <c r="J22" s="6" t="inlineStr">
         <is>
@@ -2383,11 +2387,7 @@
         </is>
       </c>
       <c r="M22" s="6" t="inlineStr"/>
-      <c r="N22" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/ortatherox/</t>
-        </is>
-      </c>
+      <c r="N22" s="6" t="inlineStr"/>
       <c r="O22" s="7" t="inlineStr"/>
       <c r="P22" s="6" t="inlineStr">
         <is>
@@ -2395,17 +2395,13 @@
         </is>
       </c>
       <c r="Q22" s="6" t="inlineStr"/>
-      <c r="R22" s="6" t="inlineStr">
-        <is>
-          <t>david@pursuit.org</t>
-        </is>
-      </c>
+      <c r="R22" s="6" t="inlineStr"/>
       <c r="S22" s="6" t="n">
-        <v>14837</v>
+        <v>6702</v>
       </c>
       <c r="T22" s="6" t="inlineStr">
         <is>
-          <t>12535</t>
+          <t>8848</t>
         </is>
       </c>
       <c r="U22" s="6" t="inlineStr">
@@ -2432,27 +2428,27 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>SHAY CPA P.C.</t>
+          <t>Stellar Health</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Akshay Shrimanker</t>
+          <t>Octavian Costache</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>Chief Executive Officer</t>
+          <t>CTO / co-founder</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>1-10</t>
+          <t>51-200</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr"/>
@@ -2480,11 +2476,11 @@
       <c r="Q23" s="6" t="inlineStr"/>
       <c r="R23" s="6" t="inlineStr"/>
       <c r="S23" s="6" t="n">
-        <v>6702</v>
+        <v>2382</v>
       </c>
       <c r="T23" s="6" t="inlineStr">
         <is>
-          <t>8848</t>
+          <t>8957</t>
         </is>
       </c>
       <c r="U23" s="6" t="inlineStr">
@@ -2511,27 +2507,27 @@
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Stellar Health</t>
+          <t>Tertulia</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Octavian Costache</t>
+          <t>Sebastian Cwilich</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>CTO / co-founder</t>
+          <t>Founder and CEO</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>51-200</t>
+          <t>1-10</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr"/>
@@ -2549,7 +2545,11 @@
         </is>
       </c>
       <c r="M24" s="6" t="inlineStr"/>
-      <c r="N24" s="6" t="inlineStr"/>
+      <c r="N24" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/sebastiancwilich</t>
+        </is>
+      </c>
       <c r="O24" s="7" t="inlineStr"/>
       <c r="P24" s="6" t="inlineStr">
         <is>
@@ -2559,11 +2559,11 @@
       <c r="Q24" s="6" t="inlineStr"/>
       <c r="R24" s="6" t="inlineStr"/>
       <c r="S24" s="6" t="n">
-        <v>2382</v>
+        <v>7156</v>
       </c>
       <c r="T24" s="6" t="inlineStr">
         <is>
-          <t>8957</t>
+          <t>9380</t>
         </is>
       </c>
       <c r="U24" s="6" t="inlineStr">
@@ -2590,33 +2590,33 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Tertulia</t>
+          <t>Alaris Capital,</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Sebastian Cwilich</t>
+          <t>Hunter Armistead</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>Founder and CEO</t>
+          <t>Chief Investment Officer</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Private Equity</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>1-10</t>
+          <t>51-200</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr"/>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K25" s="6" t="n">
@@ -2624,13 +2624,13 @@
       </c>
       <c r="L25" s="7" t="inlineStr">
         <is>
-          <t>David Yang</t>
+          <t>Joanna Patterson</t>
         </is>
       </c>
       <c r="M25" s="6" t="inlineStr"/>
       <c r="N25" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/sebastiancwilich</t>
+          <t>https://www.linkedin.com/in/hunter-armistead-61166750</t>
         </is>
       </c>
       <c r="O25" s="7" t="inlineStr"/>
@@ -2642,11 +2642,11 @@
       <c r="Q25" s="6" t="inlineStr"/>
       <c r="R25" s="6" t="inlineStr"/>
       <c r="S25" s="6" t="n">
-        <v>7156</v>
+        <v>8819</v>
       </c>
       <c r="T25" s="6" t="inlineStr">
         <is>
-          <t>9380</t>
+          <t>2462</t>
         </is>
       </c>
       <c r="U25" s="6" t="inlineStr">
@@ -2673,27 +2673,27 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Alaris Capital,</t>
+          <t>CFO Worx</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Hunter Armistead</t>
+          <t>Brian Alvarez</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Chief Investment Officer</t>
+          <t>Chief Executive Officer</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Private Equity</t>
+          <t>Consulting</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>51-200</t>
+          <t>11-50</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr"/>
@@ -2713,7 +2713,7 @@
       <c r="M26" s="6" t="inlineStr"/>
       <c r="N26" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/hunter-armistead-61166750</t>
+          <t>https://www.linkedin.com/in/briancalvarez</t>
         </is>
       </c>
       <c r="O26" s="7" t="inlineStr"/>
@@ -2725,11 +2725,11 @@
       <c r="Q26" s="6" t="inlineStr"/>
       <c r="R26" s="6" t="inlineStr"/>
       <c r="S26" s="6" t="n">
-        <v>8819</v>
+        <v>9496</v>
       </c>
       <c r="T26" s="6" t="inlineStr">
         <is>
-          <t>2462</t>
+          <t>3807</t>
         </is>
       </c>
       <c r="U26" s="6" t="inlineStr">
@@ -2756,17 +2756,17 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>CFO Worx</t>
+          <t>Digital Reach Agency</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Brian Alvarez</t>
+          <t>Andrew Seidman</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>Chief Executive Officer</t>
+          <t>COO, Co-Founder</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
@@ -2796,7 +2796,7 @@
       <c r="M27" s="6" t="inlineStr"/>
       <c r="N27" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/briancalvarez</t>
+          <t>https://www.linkedin.com/in/andrew-seidman-b555a11b</t>
         </is>
       </c>
       <c r="O27" s="7" t="inlineStr"/>
@@ -2808,11 +2808,11 @@
       <c r="Q27" s="6" t="inlineStr"/>
       <c r="R27" s="6" t="inlineStr"/>
       <c r="S27" s="6" t="n">
-        <v>9496</v>
+        <v>9796</v>
       </c>
       <c r="T27" s="6" t="inlineStr">
         <is>
-          <t>3807</t>
+          <t>4698</t>
         </is>
       </c>
       <c r="U27" s="6" t="inlineStr">
@@ -2839,22 +2839,22 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Digital Reach Agency</t>
+          <t>Ellacard</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Andrew Seidman</t>
+          <t>Francesco Balestra</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>COO, Co-Founder</t>
+          <t>Co-Founder and CEO</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>Consulting</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
@@ -2879,7 +2879,7 @@
       <c r="M28" s="6" t="inlineStr"/>
       <c r="N28" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/andrew-seidman-b555a11b</t>
+          <t>https://www.linkedin.com/in/francescobalestra</t>
         </is>
       </c>
       <c r="O28" s="7" t="inlineStr"/>
@@ -2891,11 +2891,11 @@
       <c r="Q28" s="6" t="inlineStr"/>
       <c r="R28" s="6" t="inlineStr"/>
       <c r="S28" s="6" t="n">
-        <v>9796</v>
+        <v>9135</v>
       </c>
       <c r="T28" s="6" t="inlineStr">
         <is>
-          <t>4698</t>
+          <t>4713</t>
         </is>
       </c>
       <c r="U28" s="6" t="inlineStr">
@@ -2922,27 +2922,27 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Ellacard</t>
+          <t>Embark Partners</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>Francesco Balestra</t>
+          <t>Michael Kahn</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>Co-Founder and CEO</t>
+          <t>Co-Founder and Partner</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Consulting</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>11-50</t>
+          <t>51-200</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr"/>
@@ -2962,7 +2962,7 @@
       <c r="M29" s="6" t="inlineStr"/>
       <c r="N29" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/francescobalestra</t>
+          <t>https://www.linkedin.com/in/michael-kahn-a7625b3b</t>
         </is>
       </c>
       <c r="O29" s="7" t="inlineStr"/>
@@ -2974,11 +2974,11 @@
       <c r="Q29" s="6" t="inlineStr"/>
       <c r="R29" s="6" t="inlineStr"/>
       <c r="S29" s="6" t="n">
-        <v>9135</v>
+        <v>9140</v>
       </c>
       <c r="T29" s="6" t="inlineStr">
         <is>
-          <t>4713</t>
+          <t>4667</t>
         </is>
       </c>
       <c r="U29" s="6" t="inlineStr">
@@ -3005,27 +3005,27 @@
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>Embark Partners</t>
+          <t>For Wellness</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>Michael Kahn</t>
+          <t>Greg Banbury</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>Co-Founder and Partner</t>
+          <t>Chief Executive Officer</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>Consulting</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>51-200</t>
+          <t>11-50</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr"/>
@@ -3045,7 +3045,7 @@
       <c r="M30" s="6" t="inlineStr"/>
       <c r="N30" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/michael-kahn-a7625b3b</t>
+          <t>https://www.linkedin.com/in/gregbanbury</t>
         </is>
       </c>
       <c r="O30" s="7" t="inlineStr"/>
@@ -3057,11 +3057,11 @@
       <c r="Q30" s="6" t="inlineStr"/>
       <c r="R30" s="6" t="inlineStr"/>
       <c r="S30" s="6" t="n">
-        <v>9140</v>
+        <v>8880</v>
       </c>
       <c r="T30" s="6" t="inlineStr">
         <is>
-          <t>4667</t>
+          <t>5319</t>
         </is>
       </c>
       <c r="U30" s="6" t="inlineStr">
@@ -3088,22 +3088,22 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>For Wellness</t>
+          <t>Glengarry Farm Finance</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>Greg Banbury</t>
+          <t>Greg Kalil</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>Chief Executive Officer</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr">
@@ -3128,7 +3128,7 @@
       <c r="M31" s="6" t="inlineStr"/>
       <c r="N31" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/gregbanbury</t>
+          <t>https://www.linkedin.com/in/greg-kalil-482337157</t>
         </is>
       </c>
       <c r="O31" s="7" t="inlineStr"/>
@@ -3140,11 +3140,11 @@
       <c r="Q31" s="6" t="inlineStr"/>
       <c r="R31" s="6" t="inlineStr"/>
       <c r="S31" s="6" t="n">
-        <v>8880</v>
+        <v>10259</v>
       </c>
       <c r="T31" s="6" t="inlineStr">
         <is>
-          <t>5319</t>
+          <t>5564</t>
         </is>
       </c>
       <c r="U31" s="6" t="inlineStr">
@@ -3171,22 +3171,22 @@
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>Glengarry Farm Finance</t>
+          <t>Impact Culture</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>Greg Kalil</t>
+          <t>Sofia Madden</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Founder</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Consulting</t>
         </is>
       </c>
       <c r="H32" s="6" t="inlineStr">
@@ -3211,7 +3211,7 @@
       <c r="M32" s="6" t="inlineStr"/>
       <c r="N32" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/greg-kalil-482337157</t>
+          <t>https://www.linkedin.com/in/sofiamadden</t>
         </is>
       </c>
       <c r="O32" s="7" t="inlineStr"/>
@@ -3223,11 +3223,11 @@
       <c r="Q32" s="6" t="inlineStr"/>
       <c r="R32" s="6" t="inlineStr"/>
       <c r="S32" s="6" t="n">
-        <v>10259</v>
+        <v>8689</v>
       </c>
       <c r="T32" s="6" t="inlineStr">
         <is>
-          <t>5564</t>
+          <t>5840</t>
         </is>
       </c>
       <c r="U32" s="6" t="inlineStr">
@@ -3254,27 +3254,27 @@
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Impact Culture</t>
+          <t>Pario Health</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Sofia Madden</t>
+          <t>Maggie Diehl</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>Founder</t>
+          <t>Co-Founder and CEO</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>Consulting</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>11-50</t>
+          <t>51-200</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr"/>
@@ -3294,7 +3294,7 @@
       <c r="M33" s="6" t="inlineStr"/>
       <c r="N33" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/sofiamadden</t>
+          <t>https://www.linkedin.com/in/maggie-diehl-6a975626</t>
         </is>
       </c>
       <c r="O33" s="7" t="inlineStr"/>
@@ -3306,11 +3306,11 @@
       <c r="Q33" s="6" t="inlineStr"/>
       <c r="R33" s="6" t="inlineStr"/>
       <c r="S33" s="6" t="n">
-        <v>8689</v>
+        <v>1150</v>
       </c>
       <c r="T33" s="6" t="inlineStr">
         <is>
-          <t>5840</t>
+          <t>7057</t>
         </is>
       </c>
       <c r="U33" s="6" t="inlineStr">
@@ -3337,27 +3337,27 @@
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Pario Health</t>
+          <t>Renterra</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Maggie Diehl</t>
+          <t>Andy Feis</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>Co-Founder and CEO</t>
+          <t>Co-Founder &amp; CEO</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>51-200</t>
+          <t>11-50</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr"/>
@@ -3377,7 +3377,7 @@
       <c r="M34" s="6" t="inlineStr"/>
       <c r="N34" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/maggie-diehl-6a975626</t>
+          <t>https://www.linkedin.com/in/andy-feis-97294898</t>
         </is>
       </c>
       <c r="O34" s="7" t="inlineStr"/>
@@ -3389,11 +3389,11 @@
       <c r="Q34" s="6" t="inlineStr"/>
       <c r="R34" s="6" t="inlineStr"/>
       <c r="S34" s="6" t="n">
-        <v>1150</v>
+        <v>8734</v>
       </c>
       <c r="T34" s="6" t="inlineStr">
         <is>
-          <t>7057</t>
+          <t>8362</t>
         </is>
       </c>
       <c r="U34" s="6" t="inlineStr">
@@ -3420,22 +3420,22 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Renterra</t>
+          <t>RGM TRANSPORT</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Andy Feis</t>
+          <t>Ryan Good</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>Co-Founder &amp; CEO</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Transportation</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr">
@@ -3460,7 +3460,7 @@
       <c r="M35" s="6" t="inlineStr"/>
       <c r="N35" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/andy-feis-97294898</t>
+          <t>https://www.linkedin.com/in/ryangood01</t>
         </is>
       </c>
       <c r="O35" s="7" t="inlineStr"/>
@@ -3472,11 +3472,11 @@
       <c r="Q35" s="6" t="inlineStr"/>
       <c r="R35" s="6" t="inlineStr"/>
       <c r="S35" s="6" t="n">
-        <v>8734</v>
+        <v>12095</v>
       </c>
       <c r="T35" s="6" t="inlineStr">
         <is>
-          <t>8362</t>
+          <t>7616</t>
         </is>
       </c>
       <c r="U35" s="6" t="inlineStr">
@@ -3503,27 +3503,27 @@
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>RGM TRANSPORT</t>
+          <t>Simple Homes</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Ryan Good</t>
+          <t>Jeff Hopfenbeck</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Founder &amp; CEO</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>11-50</t>
+          <t>51-200</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr"/>
@@ -3543,7 +3543,7 @@
       <c r="M36" s="6" t="inlineStr"/>
       <c r="N36" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/ryangood01</t>
+          <t>https://www.linkedin.com/in/jeffreyhopfenbeck</t>
         </is>
       </c>
       <c r="O36" s="7" t="inlineStr"/>
@@ -3555,11 +3555,11 @@
       <c r="Q36" s="6" t="inlineStr"/>
       <c r="R36" s="6" t="inlineStr"/>
       <c r="S36" s="6" t="n">
-        <v>12095</v>
+        <v>9340</v>
       </c>
       <c r="T36" s="6" t="inlineStr">
         <is>
-          <t>7616</t>
+          <t>8906</t>
         </is>
       </c>
       <c r="U36" s="6" t="inlineStr">
@@ -3586,27 +3586,27 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Simple Homes</t>
+          <t>Supermind</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Jeff Hopfenbeck</t>
+          <t>Chad Olin</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>Founder &amp; CEO</t>
+          <t>CEO &amp; Co-Founder</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>51-200</t>
+          <t>11-50</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr"/>
@@ -3626,7 +3626,7 @@
       <c r="M37" s="6" t="inlineStr"/>
       <c r="N37" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/jeffreyhopfenbeck</t>
+          <t>https://www.linkedin.com/in/chad-olin</t>
         </is>
       </c>
       <c r="O37" s="7" t="inlineStr"/>
@@ -3638,11 +3638,11 @@
       <c r="Q37" s="6" t="inlineStr"/>
       <c r="R37" s="6" t="inlineStr"/>
       <c r="S37" s="6" t="n">
-        <v>9340</v>
+        <v>9383</v>
       </c>
       <c r="T37" s="6" t="inlineStr">
         <is>
-          <t>8906</t>
+          <t>9072</t>
         </is>
       </c>
       <c r="U37" s="6" t="inlineStr">
@@ -3669,27 +3669,27 @@
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>Supermind</t>
+          <t>The Bus Network</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Chad Olin</t>
+          <t>Kyle DeVivo</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>CEO &amp; Co-Founder</t>
+          <t>Co-Founder</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Transportation</t>
         </is>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>11-50</t>
+          <t>1001-5000</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr"/>
@@ -3709,7 +3709,7 @@
       <c r="M38" s="6" t="inlineStr"/>
       <c r="N38" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/chad-olin</t>
+          <t>https://www.linkedin.com/in/kyle-devivo-2b16b845</t>
         </is>
       </c>
       <c r="O38" s="7" t="inlineStr"/>
@@ -3721,11 +3721,11 @@
       <c r="Q38" s="6" t="inlineStr"/>
       <c r="R38" s="6" t="inlineStr"/>
       <c r="S38" s="6" t="n">
-        <v>9383</v>
+        <v>9084</v>
       </c>
       <c r="T38" s="6" t="inlineStr">
         <is>
-          <t>9072</t>
+          <t>9147</t>
         </is>
       </c>
       <c r="U38" s="6" t="inlineStr">
@@ -3752,17 +3752,17 @@
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>The Bus Network</t>
+          <t>Triple Axle</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>Kyle DeVivo</t>
+          <t>Christian Battaglia</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>Co-Founder</t>
+          <t>Founder &amp; CEO</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
@@ -3772,7 +3772,7 @@
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>1001-5000</t>
+          <t>11-50</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr"/>
@@ -3790,11 +3790,7 @@
         </is>
       </c>
       <c r="M39" s="6" t="inlineStr"/>
-      <c r="N39" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/kyle-devivo-2b16b845</t>
-        </is>
-      </c>
+      <c r="N39" s="6" t="inlineStr"/>
       <c r="O39" s="7" t="inlineStr"/>
       <c r="P39" s="6" t="inlineStr">
         <is>
@@ -3804,11 +3800,11 @@
       <c r="Q39" s="6" t="inlineStr"/>
       <c r="R39" s="6" t="inlineStr"/>
       <c r="S39" s="6" t="n">
-        <v>9084</v>
+        <v>8871</v>
       </c>
       <c r="T39" s="6" t="inlineStr">
         <is>
-          <t>9147</t>
+          <t>9984</t>
         </is>
       </c>
       <c r="U39" s="6" t="inlineStr">
@@ -3835,22 +3831,22 @@
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>Triple Axle</t>
+          <t>Twain Capital</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>Christian Battaglia</t>
+          <t>David Davis</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>Founder &amp; CEO</t>
+          <t>Co-Founder and Partner</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="H40" s="6" t="inlineStr">
@@ -3873,7 +3869,11 @@
         </is>
       </c>
       <c r="M40" s="6" t="inlineStr"/>
-      <c r="N40" s="6" t="inlineStr"/>
+      <c r="N40" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/david-davis-87139812</t>
+        </is>
+      </c>
       <c r="O40" s="7" t="inlineStr"/>
       <c r="P40" s="6" t="inlineStr">
         <is>
@@ -3883,11 +3883,11 @@
       <c r="Q40" s="6" t="inlineStr"/>
       <c r="R40" s="6" t="inlineStr"/>
       <c r="S40" s="6" t="n">
-        <v>8871</v>
+        <v>9233</v>
       </c>
       <c r="T40" s="6" t="inlineStr">
         <is>
-          <t>9984</t>
+          <t>10085</t>
         </is>
       </c>
       <c r="U40" s="6" t="inlineStr">
@@ -3914,22 +3914,22 @@
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>Twain Capital</t>
+          <t>VANA Partners</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>David Davis</t>
+          <t>Chuchu J Ajukwu</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>Co-Founder and Partner</t>
+          <t>Co-Managing Partner</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Consulting</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr">
@@ -3954,7 +3954,7 @@
       <c r="M41" s="6" t="inlineStr"/>
       <c r="N41" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/david-davis-87139812</t>
+          <t>https://www.linkedin.com/in/chuchu-j-ajukwu-34ba828</t>
         </is>
       </c>
       <c r="O41" s="7" t="inlineStr"/>
@@ -3966,11 +3966,11 @@
       <c r="Q41" s="6" t="inlineStr"/>
       <c r="R41" s="6" t="inlineStr"/>
       <c r="S41" s="6" t="n">
-        <v>9233</v>
+        <v>5555</v>
       </c>
       <c r="T41" s="6" t="inlineStr">
         <is>
-          <t>10085</t>
+          <t>10145</t>
         </is>
       </c>
       <c r="U41" s="6" t="inlineStr">
@@ -3997,17 +3997,17 @@
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>VANA Partners</t>
+          <t>WhiteHorn Partners</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>Chuchu J Ajukwu</t>
+          <t>Taylor Babcock</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>Co-Managing Partner</t>
+          <t>Co-Founder</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
@@ -4017,7 +4017,7 @@
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>11-50</t>
+          <t>51-200</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr"/>
@@ -4037,7 +4037,7 @@
       <c r="M42" s="6" t="inlineStr"/>
       <c r="N42" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/chuchu-j-ajukwu-34ba828</t>
+          <t>https://www.linkedin.com/in/taylor-babcock-cfa-1b410918</t>
         </is>
       </c>
       <c r="O42" s="7" t="inlineStr"/>
@@ -4049,11 +4049,11 @@
       <c r="Q42" s="6" t="inlineStr"/>
       <c r="R42" s="6" t="inlineStr"/>
       <c r="S42" s="6" t="n">
-        <v>5555</v>
+        <v>8248</v>
       </c>
       <c r="T42" s="6" t="inlineStr">
         <is>
-          <t>10145</t>
+          <t>10644</t>
         </is>
       </c>
       <c r="U42" s="6" t="inlineStr">
@@ -4063,83 +4063,87 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="inlineStr">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="C43" s="6" t="inlineStr">
-        <is>
-          <t>Unknown — company not enriched</t>
-        </is>
-      </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>WhiteHorn Partners</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="inlineStr">
-        <is>
-          <t>Taylor Babcock</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="inlineStr">
-        <is>
-          <t>Co-Founder</t>
-        </is>
-      </c>
-      <c r="G43" s="6" t="inlineStr">
-        <is>
-          <t>Consulting</t>
-        </is>
-      </c>
-      <c r="H43" s="6" t="inlineStr">
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>No — wrong size or geo</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Artists Mutual</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Sam Mandel</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>Nonprofit</t>
+        </is>
+      </c>
+      <c r="H43" s="8" t="inlineStr">
         <is>
           <t>51-200</t>
         </is>
       </c>
-      <c r="I43" s="6" t="inlineStr"/>
-      <c r="J43" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K43" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="L43" s="7" t="inlineStr">
-        <is>
-          <t>Joanna Patterson</t>
-        </is>
-      </c>
-      <c r="M43" s="6" t="inlineStr"/>
-      <c r="N43" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/taylor-babcock-cfa-1b410918</t>
-        </is>
-      </c>
-      <c r="O43" s="7" t="inlineStr"/>
-      <c r="P43" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="Q43" s="6" t="inlineStr"/>
-      <c r="R43" s="6" t="inlineStr"/>
-      <c r="S43" s="6" t="n">
-        <v>8248</v>
-      </c>
-      <c r="T43" s="6" t="inlineStr">
-        <is>
-          <t>10644</t>
-        </is>
-      </c>
-      <c r="U43" s="6" t="inlineStr">
+      <c r="I43" s="8" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="J43" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K43" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L43" s="9" t="inlineStr">
+        <is>
+          <t>David Yang</t>
+        </is>
+      </c>
+      <c r="M43" s="8" t="inlineStr"/>
+      <c r="N43" s="8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/sammandel</t>
+        </is>
+      </c>
+      <c r="O43" s="9" t="inlineStr"/>
+      <c r="P43" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="Q43" s="8" t="inlineStr"/>
+      <c r="R43" s="8" t="inlineStr"/>
+      <c r="S43" s="8" t="n">
+        <v>2352</v>
+      </c>
+      <c r="T43" s="8" t="inlineStr">
+        <is>
+          <t>2877</t>
+        </is>
+      </c>
+      <c r="U43" s="8" t="inlineStr">
         <is>
           <t>Operation 35 — LT (Joanna / Dave)</t>
         </is>
@@ -4163,32 +4167,32 @@
       </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>Artists Mutual</t>
+          <t>Authentic Brands Group</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
-          <t>Sam Mandel</t>
+          <t>Adam Lilly</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
         <is>
-          <t>Founder</t>
+          <t>Vice President Global Marketing</t>
         </is>
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>Nonprofit</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="H44" s="8" t="inlineStr">
         <is>
-          <t>51-200</t>
+          <t>1001-5000</t>
         </is>
       </c>
       <c r="I44" s="8" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="J44" s="8" t="inlineStr">
@@ -4207,7 +4211,7 @@
       <c r="M44" s="8" t="inlineStr"/>
       <c r="N44" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/sammandel</t>
+          <t>https://www.linkedin.com/in/adamlilly</t>
         </is>
       </c>
       <c r="O44" s="9" t="inlineStr"/>
@@ -4219,11 +4223,11 @@
       <c r="Q44" s="8" t="inlineStr"/>
       <c r="R44" s="8" t="inlineStr"/>
       <c r="S44" s="8" t="n">
-        <v>2352</v>
+        <v>11200</v>
       </c>
       <c r="T44" s="8" t="inlineStr">
         <is>
-          <t>2877</t>
+          <t>3302</t>
         </is>
       </c>
       <c r="U44" s="8" t="inlineStr">
@@ -4250,32 +4254,32 @@
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>Authentic Brands Group</t>
+          <t>GOBY (www.goby.co)</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>Adam Lilly</t>
+          <t>Benjamin Goldberg</t>
         </is>
       </c>
       <c r="F45" s="8" t="inlineStr">
         <is>
-          <t>Vice President Global Marketing</t>
+          <t>Founder and CEO</t>
         </is>
       </c>
       <c r="G45" s="8" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="H45" s="8" t="inlineStr">
         <is>
-          <t>1001-5000</t>
+          <t>51-200</t>
         </is>
       </c>
       <c r="I45" s="8" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="J45" s="8" t="inlineStr">
@@ -4294,7 +4298,7 @@
       <c r="M45" s="8" t="inlineStr"/>
       <c r="N45" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/adamlilly</t>
+          <t>https://www.linkedin.com/in/bgoldberg3</t>
         </is>
       </c>
       <c r="O45" s="9" t="inlineStr"/>
@@ -4306,11 +4310,11 @@
       <c r="Q45" s="8" t="inlineStr"/>
       <c r="R45" s="8" t="inlineStr"/>
       <c r="S45" s="8" t="n">
-        <v>11200</v>
+        <v>6548</v>
       </c>
       <c r="T45" s="8" t="inlineStr">
         <is>
-          <t>3302</t>
+          <t>5578</t>
         </is>
       </c>
       <c r="U45" s="8" t="inlineStr">
@@ -4327,7 +4331,7 @@
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>Unassigned</t>
+          <t>Avni</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
@@ -4337,32 +4341,32 @@
       </c>
       <c r="D46" s="8" t="inlineStr">
         <is>
-          <t>GOBY (www.goby.co)</t>
+          <t>Kaplan</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>Benjamin Goldberg</t>
+          <t>Isaac Botier</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t>Founder and CEO</t>
+          <t>Vice President, Innovation &amp; Advising</t>
         </is>
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="H46" s="8" t="inlineStr">
         <is>
-          <t>51-200</t>
+          <t>5000+</t>
         </is>
       </c>
       <c r="I46" s="8" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="J46" s="8" t="inlineStr">
@@ -4378,10 +4382,14 @@
           <t>David Yang</t>
         </is>
       </c>
-      <c r="M46" s="8" t="inlineStr"/>
+      <c r="M46" s="8" t="inlineStr">
+        <is>
+          <t>isaac@hataragroup.com</t>
+        </is>
+      </c>
       <c r="N46" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/bgoldberg3</t>
+          <t>https://www.linkedin.com/in/isaacbotier</t>
         </is>
       </c>
       <c r="O46" s="9" t="inlineStr"/>
@@ -4391,13 +4399,17 @@
         </is>
       </c>
       <c r="Q46" s="8" t="inlineStr"/>
-      <c r="R46" s="8" t="inlineStr"/>
+      <c r="R46" s="8" t="inlineStr">
+        <is>
+          <t>avni@pursuit.org</t>
+        </is>
+      </c>
       <c r="S46" s="8" t="n">
-        <v>6548</v>
+        <v>6590</v>
       </c>
       <c r="T46" s="8" t="inlineStr">
         <is>
-          <t>5578</t>
+          <t>6519</t>
         </is>
       </c>
       <c r="U46" s="8" t="inlineStr">
@@ -4414,7 +4426,7 @@
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>Avni</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
@@ -4424,32 +4436,32 @@
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>Kaplan</t>
+          <t>Lightmatter</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>Isaac Botier</t>
+          <t>Greg Hausheer</t>
         </is>
       </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
-          <t>Vice President, Innovation &amp; Advising</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="G47" s="8" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="H47" s="8" t="inlineStr">
         <is>
-          <t>5000+</t>
+          <t>51-200</t>
         </is>
       </c>
       <c r="I47" s="8" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="J47" s="8" t="inlineStr">
@@ -4465,14 +4477,10 @@
           <t>David Yang</t>
         </is>
       </c>
-      <c r="M47" s="8" t="inlineStr">
-        <is>
-          <t>isaac@hataragroup.com</t>
-        </is>
-      </c>
+      <c r="M47" s="8" t="inlineStr"/>
       <c r="N47" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/isaacbotier</t>
+          <t>https://www.linkedin.com/in/greghausheer</t>
         </is>
       </c>
       <c r="O47" s="9" t="inlineStr"/>
@@ -4482,17 +4490,13 @@
         </is>
       </c>
       <c r="Q47" s="8" t="inlineStr"/>
-      <c r="R47" s="8" t="inlineStr">
-        <is>
-          <t>avni@pursuit.org</t>
-        </is>
-      </c>
+      <c r="R47" s="8" t="inlineStr"/>
       <c r="S47" s="8" t="n">
-        <v>6590</v>
+        <v>7273</v>
       </c>
       <c r="T47" s="8" t="inlineStr">
         <is>
-          <t>6519</t>
+          <t>6023</t>
         </is>
       </c>
       <c r="U47" s="8" t="inlineStr">
@@ -4519,32 +4523,32 @@
       </c>
       <c r="D48" s="8" t="inlineStr">
         <is>
-          <t>Lightmatter</t>
+          <t>Major League Hacking</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
         <is>
-          <t>Greg Hausheer</t>
+          <t>💻 Jonathan Gottfried</t>
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Co-Founder</t>
         </is>
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="H48" s="8" t="inlineStr">
         <is>
-          <t>51-200</t>
+          <t>11-50</t>
         </is>
       </c>
       <c r="I48" s="8" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="J48" s="8" t="inlineStr">
@@ -4561,11 +4565,7 @@
         </is>
       </c>
       <c r="M48" s="8" t="inlineStr"/>
-      <c r="N48" s="8" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/greghausheer</t>
-        </is>
-      </c>
+      <c r="N48" s="8" t="inlineStr"/>
       <c r="O48" s="9" t="inlineStr"/>
       <c r="P48" s="8" t="inlineStr">
         <is>
@@ -4575,11 +4575,11 @@
       <c r="Q48" s="8" t="inlineStr"/>
       <c r="R48" s="8" t="inlineStr"/>
       <c r="S48" s="8" t="n">
-        <v>7273</v>
+        <v>6704</v>
       </c>
       <c r="T48" s="8" t="inlineStr">
         <is>
-          <t>6023</t>
+          <t>6453</t>
         </is>
       </c>
       <c r="U48" s="8" t="inlineStr">
@@ -4606,22 +4606,22 @@
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>Major League Hacking</t>
+          <t>mRelief</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>💻 Jonathan Gottfried</t>
+          <t>Genevieve Nielsen</t>
         </is>
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
-          <t>Co-Founder</t>
+          <t>Co-Founder and Board Member</t>
         </is>
       </c>
       <c r="G49" s="8" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Nonprofit</t>
         </is>
       </c>
       <c r="H49" s="8" t="inlineStr">
@@ -4631,7 +4631,7 @@
       </c>
       <c r="I49" s="8" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="J49" s="8" t="inlineStr">
@@ -4648,7 +4648,11 @@
         </is>
       </c>
       <c r="M49" s="8" t="inlineStr"/>
-      <c r="N49" s="8" t="inlineStr"/>
+      <c r="N49" s="8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/genevievenielsen</t>
+        </is>
+      </c>
       <c r="O49" s="9" t="inlineStr"/>
       <c r="P49" s="8" t="inlineStr">
         <is>
@@ -4658,11 +4662,11 @@
       <c r="Q49" s="8" t="inlineStr"/>
       <c r="R49" s="8" t="inlineStr"/>
       <c r="S49" s="8" t="n">
-        <v>6704</v>
+        <v>7209</v>
       </c>
       <c r="T49" s="8" t="inlineStr">
         <is>
-          <t>6453</t>
+          <t>7731</t>
         </is>
       </c>
       <c r="U49" s="8" t="inlineStr">
@@ -4689,32 +4693,32 @@
       </c>
       <c r="D50" s="8" t="inlineStr">
         <is>
-          <t>mRelief</t>
+          <t>Notion</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr">
         <is>
-          <t>Genevieve Nielsen</t>
+          <t>Alan Johnson</t>
         </is>
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t>Co-Founder and Board Member</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>Nonprofit</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="H50" s="8" t="inlineStr">
         <is>
-          <t>11-50</t>
+          <t>201-1000</t>
         </is>
       </c>
       <c r="I50" s="8" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="J50" s="8" t="inlineStr">
@@ -4731,11 +4735,7 @@
         </is>
       </c>
       <c r="M50" s="8" t="inlineStr"/>
-      <c r="N50" s="8" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/genevievenielsen</t>
-        </is>
-      </c>
+      <c r="N50" s="8" t="inlineStr"/>
       <c r="O50" s="9" t="inlineStr"/>
       <c r="P50" s="8" t="inlineStr">
         <is>
@@ -4745,11 +4745,11 @@
       <c r="Q50" s="8" t="inlineStr"/>
       <c r="R50" s="8" t="inlineStr"/>
       <c r="S50" s="8" t="n">
-        <v>7209</v>
+        <v>15151</v>
       </c>
       <c r="T50" s="8" t="inlineStr">
         <is>
-          <t>7731</t>
+          <t>12439</t>
         </is>
       </c>
       <c r="U50" s="8" t="inlineStr">
@@ -4776,32 +4776,32 @@
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>Notion</t>
+          <t>RXR</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t>Alan Johnson</t>
+          <t>Adam Greene</t>
         </is>
       </c>
       <c r="F51" s="8" t="inlineStr">
         <is>
-          <t>Software Engineer</t>
+          <t>Senior Vice President, Development</t>
         </is>
       </c>
       <c r="G51" s="8" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="H51" s="8" t="inlineStr">
         <is>
-          <t>201-1000</t>
+          <t>1001-5000</t>
         </is>
       </c>
       <c r="I51" s="8" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="J51" s="8" t="inlineStr">
@@ -4818,7 +4818,11 @@
         </is>
       </c>
       <c r="M51" s="8" t="inlineStr"/>
-      <c r="N51" s="8" t="inlineStr"/>
+      <c r="N51" s="8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/greeneadam</t>
+        </is>
+      </c>
       <c r="O51" s="9" t="inlineStr"/>
       <c r="P51" s="8" t="inlineStr">
         <is>
@@ -4828,11 +4832,11 @@
       <c r="Q51" s="8" t="inlineStr"/>
       <c r="R51" s="8" t="inlineStr"/>
       <c r="S51" s="8" t="n">
-        <v>15151</v>
+        <v>6779</v>
       </c>
       <c r="T51" s="8" t="inlineStr">
         <is>
-          <t>12439</t>
+          <t>1665</t>
         </is>
       </c>
       <c r="U51" s="8" t="inlineStr">
@@ -4859,37 +4863,37 @@
       </c>
       <c r="D52" s="8" t="inlineStr">
         <is>
-          <t>RXR</t>
+          <t>Alara Imaging</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr">
         <is>
-          <t>Adam Greene</t>
+          <t>Nate Mazonson</t>
         </is>
       </c>
       <c r="F52" s="8" t="inlineStr">
         <is>
-          <t>Senior Vice President, Development</t>
+          <t>Co-Founder and CEO</t>
         </is>
       </c>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="H52" s="8" t="inlineStr">
         <is>
-          <t>1001-5000</t>
+          <t>51-200</t>
         </is>
       </c>
       <c r="I52" s="8" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>null</t>
         </is>
       </c>
       <c r="J52" s="8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K52" s="8" t="n">
@@ -4897,13 +4901,13 @@
       </c>
       <c r="L52" s="9" t="inlineStr">
         <is>
-          <t>David Yang</t>
+          <t>Joanna Patterson</t>
         </is>
       </c>
       <c r="M52" s="8" t="inlineStr"/>
       <c r="N52" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/greeneadam</t>
+          <t>https://www.linkedin.com/in/mazonson</t>
         </is>
       </c>
       <c r="O52" s="9" t="inlineStr"/>
@@ -4915,11 +4919,11 @@
       <c r="Q52" s="8" t="inlineStr"/>
       <c r="R52" s="8" t="inlineStr"/>
       <c r="S52" s="8" t="n">
-        <v>6779</v>
+        <v>9614</v>
       </c>
       <c r="T52" s="8" t="inlineStr">
         <is>
-          <t>1665</t>
+          <t>2756</t>
         </is>
       </c>
       <c r="U52" s="8" t="inlineStr">
@@ -4946,27 +4950,27 @@
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>Alara Imaging</t>
+          <t>AmericanStar Trailways</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
         <is>
-          <t>Nate Mazonson</t>
+          <t>Roni Alvandi</t>
         </is>
       </c>
       <c r="F53" s="8" t="inlineStr">
         <is>
-          <t>Co-Founder and CEO</t>
+          <t>President and CEO</t>
         </is>
       </c>
       <c r="G53" s="8" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Transportation</t>
         </is>
       </c>
       <c r="H53" s="8" t="inlineStr">
         <is>
-          <t>51-200</t>
+          <t>201-1000</t>
         </is>
       </c>
       <c r="I53" s="8" t="inlineStr">
@@ -4990,7 +4994,7 @@
       <c r="M53" s="8" t="inlineStr"/>
       <c r="N53" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mazonson</t>
+          <t>https://www.linkedin.com/in/roni-alvandi-9207b6178</t>
         </is>
       </c>
       <c r="O53" s="9" t="inlineStr"/>
@@ -5002,11 +5006,11 @@
       <c r="Q53" s="8" t="inlineStr"/>
       <c r="R53" s="8" t="inlineStr"/>
       <c r="S53" s="8" t="n">
-        <v>9614</v>
+        <v>9089</v>
       </c>
       <c r="T53" s="8" t="inlineStr">
         <is>
-          <t>2756</t>
+          <t>2634</t>
         </is>
       </c>
       <c r="U53" s="8" t="inlineStr">
@@ -5033,32 +5037,32 @@
       </c>
       <c r="D54" s="8" t="inlineStr">
         <is>
-          <t>AmericanStar Trailways</t>
+          <t>August Schools</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
         <is>
-          <t>Roni Alvandi</t>
+          <t>Peter Russell</t>
         </is>
       </c>
       <c r="F54" s="8" t="inlineStr">
         <is>
-          <t>President and CEO</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="G54" s="8" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="H54" s="8" t="inlineStr">
         <is>
-          <t>201-1000</t>
+          <t>51-200</t>
         </is>
       </c>
       <c r="I54" s="8" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="J54" s="8" t="inlineStr">
@@ -5077,7 +5081,7 @@
       <c r="M54" s="8" t="inlineStr"/>
       <c r="N54" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/roni-alvandi-9207b6178</t>
+          <t>https://www.linkedin.com/in/mrpeterrussell</t>
         </is>
       </c>
       <c r="O54" s="9" t="inlineStr"/>
@@ -5089,11 +5093,11 @@
       <c r="Q54" s="8" t="inlineStr"/>
       <c r="R54" s="8" t="inlineStr"/>
       <c r="S54" s="8" t="n">
-        <v>9089</v>
+        <v>8851</v>
       </c>
       <c r="T54" s="8" t="inlineStr">
         <is>
-          <t>2634</t>
+          <t>3301</t>
         </is>
       </c>
       <c r="U54" s="8" t="inlineStr">
@@ -5120,32 +5124,32 @@
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>August Schools</t>
+          <t>Black Creek Digital</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t>Peter Russell</t>
+          <t>Chris Lawlor</t>
         </is>
       </c>
       <c r="F55" s="8" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Co-Founder and Chief Product Officer</t>
         </is>
       </c>
       <c r="G55" s="8" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="H55" s="8" t="inlineStr">
         <is>
-          <t>51-200</t>
+          <t>1001-5000</t>
         </is>
       </c>
       <c r="I55" s="8" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>Jacksonville, FL</t>
         </is>
       </c>
       <c r="J55" s="8" t="inlineStr">
@@ -5162,11 +5166,7 @@
         </is>
       </c>
       <c r="M55" s="8" t="inlineStr"/>
-      <c r="N55" s="8" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/mrpeterrussell</t>
-        </is>
-      </c>
+      <c r="N55" s="8" t="inlineStr"/>
       <c r="O55" s="9" t="inlineStr"/>
       <c r="P55" s="8" t="inlineStr">
         <is>
@@ -5176,11 +5176,11 @@
       <c r="Q55" s="8" t="inlineStr"/>
       <c r="R55" s="8" t="inlineStr"/>
       <c r="S55" s="8" t="n">
-        <v>8851</v>
+        <v>12590</v>
       </c>
       <c r="T55" s="8" t="inlineStr">
         <is>
-          <t>3301</t>
+          <t>9576</t>
         </is>
       </c>
       <c r="U55" s="8" t="inlineStr">
@@ -5207,32 +5207,32 @@
       </c>
       <c r="D56" s="8" t="inlineStr">
         <is>
-          <t>Black Creek Digital</t>
+          <t>Boost My School</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
         <is>
-          <t>Chris Lawlor</t>
+          <t>Holman Gao</t>
         </is>
       </c>
       <c r="F56" s="8" t="inlineStr">
         <is>
-          <t>Co-Founder and Chief Product Officer</t>
+          <t>CEO &amp; Founder</t>
         </is>
       </c>
       <c r="G56" s="8" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="H56" s="8" t="inlineStr">
         <is>
-          <t>1001-5000</t>
+          <t>11-50</t>
         </is>
       </c>
       <c r="I56" s="8" t="inlineStr">
         <is>
-          <t>Jacksonville, FL</t>
+          <t>Unknown, Unknown</t>
         </is>
       </c>
       <c r="J56" s="8" t="inlineStr">
@@ -5249,7 +5249,11 @@
         </is>
       </c>
       <c r="M56" s="8" t="inlineStr"/>
-      <c r="N56" s="8" t="inlineStr"/>
+      <c r="N56" s="8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/holman-gao</t>
+        </is>
+      </c>
       <c r="O56" s="9" t="inlineStr"/>
       <c r="P56" s="8" t="inlineStr">
         <is>
@@ -5259,11 +5263,11 @@
       <c r="Q56" s="8" t="inlineStr"/>
       <c r="R56" s="8" t="inlineStr"/>
       <c r="S56" s="8" t="n">
-        <v>12590</v>
+        <v>8654</v>
       </c>
       <c r="T56" s="8" t="inlineStr">
         <is>
-          <t>9576</t>
+          <t>3042</t>
         </is>
       </c>
       <c r="U56" s="8" t="inlineStr">
@@ -5290,12 +5294,12 @@
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>Boost My School</t>
+          <t>cred.</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t>Holman Gao</t>
+          <t>Caitlin Bartley (Caitlin MacDonald)</t>
         </is>
       </c>
       <c r="F57" s="8" t="inlineStr">
@@ -5305,17 +5309,17 @@
       </c>
       <c r="G57" s="8" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="H57" s="8" t="inlineStr">
         <is>
-          <t>11-50</t>
+          <t>201-1000</t>
         </is>
       </c>
       <c r="I57" s="8" t="inlineStr">
         <is>
-          <t>Unknown, Unknown</t>
+          <t>Mumbai, India</t>
         </is>
       </c>
       <c r="J57" s="8" t="inlineStr">
@@ -5334,7 +5338,7 @@
       <c r="M57" s="8" t="inlineStr"/>
       <c r="N57" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/holman-gao</t>
+          <t>https://www.linkedin.com/in/caitlinabartley</t>
         </is>
       </c>
       <c r="O57" s="9" t="inlineStr"/>
@@ -5346,11 +5350,11 @@
       <c r="Q57" s="8" t="inlineStr"/>
       <c r="R57" s="8" t="inlineStr"/>
       <c r="S57" s="8" t="n">
-        <v>8654</v>
+        <v>9920</v>
       </c>
       <c r="T57" s="8" t="inlineStr">
         <is>
-          <t>3042</t>
+          <t>4166</t>
         </is>
       </c>
       <c r="U57" s="8" t="inlineStr">
@@ -5367,7 +5371,7 @@
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>Devika</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
@@ -5377,32 +5381,32 @@
       </c>
       <c r="D58" s="8" t="inlineStr">
         <is>
-          <t>Con Edison</t>
+          <t>CueBox</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
         <is>
-          <t>Jen Hensley</t>
+          <t>Christina Pan</t>
         </is>
       </c>
       <c r="F58" s="8" t="inlineStr">
         <is>
-          <t>Senior Vice President, Corporate Affairs</t>
+          <t>CEO &amp; Co-Founder @ CueBox</t>
         </is>
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>5000+</t>
+          <t>11-50</t>
         </is>
       </c>
       <c r="I58" s="8" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="J58" s="8" t="inlineStr">
@@ -5415,17 +5419,13 @@
       </c>
       <c r="L58" s="9" t="inlineStr">
         <is>
-          <t>David Yang</t>
-        </is>
-      </c>
-      <c r="M58" s="8" t="inlineStr">
-        <is>
-          <t>hensleyj@coned.com</t>
-        </is>
-      </c>
+          <t>Joanna Patterson</t>
+        </is>
+      </c>
+      <c r="M58" s="8" t="inlineStr"/>
       <c r="N58" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/jen-hensley</t>
+          <t>https://www.linkedin.com/in/christina-pan-469a7319</t>
         </is>
       </c>
       <c r="O58" s="9" t="inlineStr"/>
@@ -5435,22 +5435,18 @@
         </is>
       </c>
       <c r="Q58" s="8" t="inlineStr"/>
-      <c r="R58" s="8" t="inlineStr">
-        <is>
-          <t>devika@pursuit.org</t>
-        </is>
-      </c>
+      <c r="R58" s="8" t="inlineStr"/>
       <c r="S58" s="8" t="n">
-        <v>11570</v>
+        <v>8692</v>
       </c>
       <c r="T58" s="8" t="inlineStr">
         <is>
-          <t>590</t>
+          <t>10197</t>
         </is>
       </c>
       <c r="U58" s="8" t="inlineStr">
         <is>
-          <t>LT_Nick list, but rated only by Joanna/Dave</t>
+          <t>Operation 35 — LT (Joanna / Dave)</t>
         </is>
       </c>
     </row>
@@ -5472,32 +5468,32 @@
       </c>
       <c r="D59" s="8" t="inlineStr">
         <is>
-          <t>cred.</t>
+          <t>Cushman &amp; Wakefield</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t>Caitlin Bartley (Caitlin MacDonald)</t>
+          <t>Michael Movshovich</t>
         </is>
       </c>
       <c r="F59" s="8" t="inlineStr">
         <is>
-          <t>CEO &amp; Founder</t>
+          <t>Vice Chairman | Head of Alternative Investment Advisory</t>
         </is>
       </c>
       <c r="G59" s="8" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="H59" s="8" t="inlineStr">
         <is>
-          <t>201-1000</t>
+          <t>5000+</t>
         </is>
       </c>
       <c r="I59" s="8" t="inlineStr">
         <is>
-          <t>Mumbai, India</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="J59" s="8" t="inlineStr">
@@ -5506,17 +5502,17 @@
         </is>
       </c>
       <c r="K59" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L59" s="9" t="inlineStr">
         <is>
-          <t>Joanna Patterson</t>
+          <t>David Yang | Victoria Mayo</t>
         </is>
       </c>
       <c r="M59" s="8" t="inlineStr"/>
       <c r="N59" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/caitlinabartley</t>
+          <t>https://www.linkedin.com/in/michael-movshovich-8691485</t>
         </is>
       </c>
       <c r="O59" s="9" t="inlineStr"/>
@@ -5528,11 +5524,11 @@
       <c r="Q59" s="8" t="inlineStr"/>
       <c r="R59" s="8" t="inlineStr"/>
       <c r="S59" s="8" t="n">
-        <v>9920</v>
+        <v>6797</v>
       </c>
       <c r="T59" s="8" t="inlineStr">
         <is>
-          <t>4166</t>
+          <t>4263</t>
         </is>
       </c>
       <c r="U59" s="8" t="inlineStr">
@@ -5559,22 +5555,22 @@
       </c>
       <c r="D60" s="8" t="inlineStr">
         <is>
-          <t>CueBox</t>
+          <t>Drawdown Fund</t>
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr">
         <is>
-          <t>Christina Pan</t>
+          <t>Erik Snyder</t>
         </is>
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t>CEO &amp; Co-Founder @ CueBox</t>
+          <t>CEO, Founder</t>
         </is>
       </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="H60" s="8" t="inlineStr">
@@ -5584,7 +5580,7 @@
       </c>
       <c r="I60" s="8" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="J60" s="8" t="inlineStr">
@@ -5603,7 +5599,7 @@
       <c r="M60" s="8" t="inlineStr"/>
       <c r="N60" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/christina-pan-469a7319</t>
+          <t>https://www.linkedin.com/in/erik-snyder-8529871</t>
         </is>
       </c>
       <c r="O60" s="9" t="inlineStr"/>
@@ -5615,11 +5611,11 @@
       <c r="Q60" s="8" t="inlineStr"/>
       <c r="R60" s="8" t="inlineStr"/>
       <c r="S60" s="8" t="n">
-        <v>8692</v>
+        <v>9499</v>
       </c>
       <c r="T60" s="8" t="inlineStr">
         <is>
-          <t>10197</t>
+          <t>4491</t>
         </is>
       </c>
       <c r="U60" s="8" t="inlineStr">
@@ -5646,17 +5642,17 @@
       </c>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>Cushman &amp; Wakefield</t>
+          <t>Gallatin Builders</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t>Michael Movshovich</t>
+          <t>JB Cholnoky</t>
         </is>
       </c>
       <c r="F61" s="8" t="inlineStr">
         <is>
-          <t>Vice Chairman | Head of Alternative Investment Advisory</t>
+          <t>Founder / Owner</t>
         </is>
       </c>
       <c r="G61" s="8" t="inlineStr">
@@ -5666,12 +5662,12 @@
       </c>
       <c r="H61" s="8" t="inlineStr">
         <is>
-          <t>5000+</t>
+          <t>51-200</t>
         </is>
       </c>
       <c r="I61" s="8" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Gallatin, MT</t>
         </is>
       </c>
       <c r="J61" s="8" t="inlineStr">
@@ -5680,17 +5676,17 @@
         </is>
       </c>
       <c r="K61" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L61" s="9" t="inlineStr">
         <is>
-          <t>David Yang | Victoria Mayo</t>
+          <t>Joanna Patterson</t>
         </is>
       </c>
       <c r="M61" s="8" t="inlineStr"/>
       <c r="N61" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/michael-movshovich-8691485</t>
+          <t>https://www.linkedin.com/in/jb-cholnoky-71655011</t>
         </is>
       </c>
       <c r="O61" s="9" t="inlineStr"/>
@@ -5702,11 +5698,11 @@
       <c r="Q61" s="8" t="inlineStr"/>
       <c r="R61" s="8" t="inlineStr"/>
       <c r="S61" s="8" t="n">
-        <v>6797</v>
+        <v>10198</v>
       </c>
       <c r="T61" s="8" t="inlineStr">
         <is>
-          <t>4263</t>
+          <t>5695</t>
         </is>
       </c>
       <c r="U61" s="8" t="inlineStr">
@@ -5733,22 +5729,22 @@
       </c>
       <c r="D62" s="8" t="inlineStr">
         <is>
-          <t>Drawdown Fund</t>
+          <t>Ilion Capital Partners</t>
         </is>
       </c>
       <c r="E62" s="8" t="inlineStr">
         <is>
-          <t>Erik Snyder</t>
+          <t>Andrew Hennessy</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t>CEO, Founder</t>
+          <t>Managing Partner</t>
         </is>
       </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Private Equity</t>
         </is>
       </c>
       <c r="H62" s="8" t="inlineStr">
@@ -5777,7 +5773,7 @@
       <c r="M62" s="8" t="inlineStr"/>
       <c r="N62" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/erik-snyder-8529871</t>
+          <t>https://www.linkedin.com/in/andrew-h-58738414</t>
         </is>
       </c>
       <c r="O62" s="9" t="inlineStr"/>
@@ -5789,11 +5785,11 @@
       <c r="Q62" s="8" t="inlineStr"/>
       <c r="R62" s="8" t="inlineStr"/>
       <c r="S62" s="8" t="n">
-        <v>9499</v>
+        <v>8997</v>
       </c>
       <c r="T62" s="8" t="inlineStr">
         <is>
-          <t>4491</t>
+          <t>5982</t>
         </is>
       </c>
       <c r="U62" s="8" t="inlineStr">
@@ -5820,32 +5816,32 @@
       </c>
       <c r="D63" s="8" t="inlineStr">
         <is>
-          <t>Gallatin Builders</t>
+          <t>Ilion Capital Partners</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t>JB Cholnoky</t>
+          <t>Jonathan Slonim</t>
         </is>
       </c>
       <c r="F63" s="8" t="inlineStr">
         <is>
-          <t>Founder / Owner</t>
+          <t>Managing Partner</t>
         </is>
       </c>
       <c r="G63" s="8" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Private Equity</t>
         </is>
       </c>
       <c r="H63" s="8" t="inlineStr">
         <is>
-          <t>51-200</t>
+          <t>11-50</t>
         </is>
       </c>
       <c r="I63" s="8" t="inlineStr">
         <is>
-          <t>Gallatin, MT</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="J63" s="8" t="inlineStr">
@@ -5864,7 +5860,7 @@
       <c r="M63" s="8" t="inlineStr"/>
       <c r="N63" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/jb-cholnoky-71655011</t>
+          <t>https://www.linkedin.com/in/jonathanslonim</t>
         </is>
       </c>
       <c r="O63" s="9" t="inlineStr"/>
@@ -5876,11 +5872,11 @@
       <c r="Q63" s="8" t="inlineStr"/>
       <c r="R63" s="8" t="inlineStr"/>
       <c r="S63" s="8" t="n">
-        <v>10198</v>
+        <v>9193</v>
       </c>
       <c r="T63" s="8" t="inlineStr">
         <is>
-          <t>5695</t>
+          <t>5982</t>
         </is>
       </c>
       <c r="U63" s="8" t="inlineStr">
@@ -5907,32 +5903,32 @@
       </c>
       <c r="D64" s="8" t="inlineStr">
         <is>
-          <t>Ilion Capital Partners</t>
+          <t>Jordan Park Group</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
         <is>
-          <t>Andrew Hennessy</t>
+          <t>Meeka Charles</t>
         </is>
       </c>
       <c r="F64" s="8" t="inlineStr">
         <is>
-          <t>Managing Partner</t>
+          <t>Vice President, Client Advisory</t>
         </is>
       </c>
       <c r="G64" s="8" t="inlineStr">
         <is>
-          <t>Private Equity</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="H64" s="8" t="inlineStr">
         <is>
-          <t>11-50</t>
+          <t>51-200</t>
         </is>
       </c>
       <c r="I64" s="8" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>null</t>
         </is>
       </c>
       <c r="J64" s="8" t="inlineStr">
@@ -5951,7 +5947,7 @@
       <c r="M64" s="8" t="inlineStr"/>
       <c r="N64" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/andrew-h-58738414</t>
+          <t>https://www.linkedin.com/in/meekacharles</t>
         </is>
       </c>
       <c r="O64" s="9" t="inlineStr"/>
@@ -5963,11 +5959,11 @@
       <c r="Q64" s="8" t="inlineStr"/>
       <c r="R64" s="8" t="inlineStr"/>
       <c r="S64" s="8" t="n">
-        <v>8997</v>
+        <v>10000</v>
       </c>
       <c r="T64" s="8" t="inlineStr">
         <is>
-          <t>5982</t>
+          <t>6306</t>
         </is>
       </c>
       <c r="U64" s="8" t="inlineStr">
@@ -5994,32 +5990,32 @@
       </c>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>Ilion Capital Partners</t>
+          <t>Juno</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>Jonathan Slonim</t>
+          <t>Jonathan Scherr</t>
         </is>
       </c>
       <c r="F65" s="8" t="inlineStr">
         <is>
-          <t>Managing Partner</t>
+          <t>Founder and CEO</t>
         </is>
       </c>
       <c r="G65" s="8" t="inlineStr">
         <is>
-          <t>Private Equity</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="H65" s="8" t="inlineStr">
         <is>
-          <t>11-50</t>
+          <t>51-200</t>
         </is>
       </c>
       <c r="I65" s="8" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="J65" s="8" t="inlineStr">
@@ -6038,7 +6034,7 @@
       <c r="M65" s="8" t="inlineStr"/>
       <c r="N65" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/jonathanslonim</t>
+          <t>https://www.linkedin.com/in/jbscherr</t>
         </is>
       </c>
       <c r="O65" s="9" t="inlineStr"/>
@@ -6050,11 +6046,11 @@
       <c r="Q65" s="8" t="inlineStr"/>
       <c r="R65" s="8" t="inlineStr"/>
       <c r="S65" s="8" t="n">
-        <v>9193</v>
+        <v>9921</v>
       </c>
       <c r="T65" s="8" t="inlineStr">
         <is>
-          <t>5982</t>
+          <t>6466</t>
         </is>
       </c>
       <c r="U65" s="8" t="inlineStr">
@@ -6081,22 +6077,22 @@
       </c>
       <c r="D66" s="8" t="inlineStr">
         <is>
-          <t>Jordan Park Group</t>
+          <t>Latin American Leadership Academy</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t>Meeka Charles</t>
+          <t>Diego Ontaneda Benavides</t>
         </is>
       </c>
       <c r="F66" s="8" t="inlineStr">
         <is>
-          <t>Vice President, Client Advisory</t>
+          <t>Co-Founder &amp; CEO</t>
         </is>
       </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="H66" s="8" t="inlineStr">
@@ -6125,7 +6121,7 @@
       <c r="M66" s="8" t="inlineStr"/>
       <c r="N66" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/meekacharles</t>
+          <t>https://www.linkedin.com/in/diegofromperu</t>
         </is>
       </c>
       <c r="O66" s="9" t="inlineStr"/>
@@ -6137,11 +6133,11 @@
       <c r="Q66" s="8" t="inlineStr"/>
       <c r="R66" s="8" t="inlineStr"/>
       <c r="S66" s="8" t="n">
-        <v>10000</v>
+        <v>1365</v>
       </c>
       <c r="T66" s="8" t="inlineStr">
         <is>
-          <t>6306</t>
+          <t>5961</t>
         </is>
       </c>
       <c r="U66" s="8" t="inlineStr">
@@ -6168,32 +6164,32 @@
       </c>
       <c r="D67" s="8" t="inlineStr">
         <is>
-          <t>Juno</t>
+          <t>Luminus Prep</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t>Jonathan Scherr</t>
+          <t>John Murphy</t>
         </is>
       </c>
       <c r="F67" s="8" t="inlineStr">
         <is>
-          <t>Founder and CEO</t>
+          <t>Co-Founder</t>
         </is>
       </c>
       <c r="G67" s="8" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="H67" s="8" t="inlineStr">
         <is>
-          <t>51-200</t>
+          <t>11-50</t>
         </is>
       </c>
       <c r="I67" s="8" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="J67" s="8" t="inlineStr">
@@ -6210,11 +6206,7 @@
         </is>
       </c>
       <c r="M67" s="8" t="inlineStr"/>
-      <c r="N67" s="8" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/jbscherr</t>
-        </is>
-      </c>
+      <c r="N67" s="8" t="inlineStr"/>
       <c r="O67" s="9" t="inlineStr"/>
       <c r="P67" s="8" t="inlineStr">
         <is>
@@ -6224,11 +6216,11 @@
       <c r="Q67" s="8" t="inlineStr"/>
       <c r="R67" s="8" t="inlineStr"/>
       <c r="S67" s="8" t="n">
-        <v>9921</v>
+        <v>12562</v>
       </c>
       <c r="T67" s="8" t="inlineStr">
         <is>
-          <t>6466</t>
+          <t>9533</t>
         </is>
       </c>
       <c r="U67" s="8" t="inlineStr">
@@ -6255,22 +6247,22 @@
       </c>
       <c r="D68" s="8" t="inlineStr">
         <is>
-          <t>Latin American Leadership Academy</t>
+          <t>Maia Oncology</t>
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t>Diego Ontaneda Benavides</t>
+          <t>Liya Shuster-Bier</t>
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t>Co-Founder &amp; CEO</t>
+          <t>Founder &amp; CEO</t>
         </is>
       </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="H68" s="8" t="inlineStr">
@@ -6280,7 +6272,7 @@
       </c>
       <c r="I68" s="8" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="J68" s="8" t="inlineStr">
@@ -6299,7 +6291,7 @@
       <c r="M68" s="8" t="inlineStr"/>
       <c r="N68" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/diegofromperu</t>
+          <t>https://www.linkedin.com/in/liyashusterbier</t>
         </is>
       </c>
       <c r="O68" s="9" t="inlineStr"/>
@@ -6311,11 +6303,11 @@
       <c r="Q68" s="8" t="inlineStr"/>
       <c r="R68" s="8" t="inlineStr"/>
       <c r="S68" s="8" t="n">
-        <v>1365</v>
+        <v>6557</v>
       </c>
       <c r="T68" s="8" t="inlineStr">
         <is>
-          <t>5961</t>
+          <t>6450</t>
         </is>
       </c>
       <c r="U68" s="8" t="inlineStr">
@@ -6342,22 +6334,22 @@
       </c>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>Luminus Prep</t>
+          <t>Moms First (formerly Marshall Plan for Moms)</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>John Murphy</t>
+          <t>Reshma Saujani</t>
         </is>
       </c>
       <c r="F69" s="8" t="inlineStr">
         <is>
-          <t>Co-Founder</t>
+          <t>Founder and CEO</t>
         </is>
       </c>
       <c r="G69" s="8" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Nonprofit</t>
         </is>
       </c>
       <c r="H69" s="8" t="inlineStr">
@@ -6380,11 +6372,15 @@
       </c>
       <c r="L69" s="9" t="inlineStr">
         <is>
-          <t>Joanna Patterson</t>
+          <t>David Yang</t>
         </is>
       </c>
       <c r="M69" s="8" t="inlineStr"/>
-      <c r="N69" s="8" t="inlineStr"/>
+      <c r="N69" s="8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/reshma-saujani</t>
+        </is>
+      </c>
       <c r="O69" s="9" t="inlineStr"/>
       <c r="P69" s="8" t="inlineStr">
         <is>
@@ -6394,11 +6390,11 @@
       <c r="Q69" s="8" t="inlineStr"/>
       <c r="R69" s="8" t="inlineStr"/>
       <c r="S69" s="8" t="n">
-        <v>12562</v>
+        <v>2342</v>
       </c>
       <c r="T69" s="8" t="inlineStr">
         <is>
-          <t>9533</t>
+          <t>7491</t>
         </is>
       </c>
       <c r="U69" s="8" t="inlineStr">
@@ -6425,32 +6421,32 @@
       </c>
       <c r="D70" s="8" t="inlineStr">
         <is>
-          <t>Maia Oncology</t>
+          <t>Nature Inc. (Nature Remo)</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr">
         <is>
-          <t>Liya Shuster-Bier</t>
+          <t>Haruumi Shiode</t>
         </is>
       </c>
       <c r="F70" s="8" t="inlineStr">
         <is>
-          <t>Founder &amp; CEO</t>
+          <t>Founder</t>
         </is>
       </c>
       <c r="G70" s="8" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="H70" s="8" t="inlineStr">
         <is>
-          <t>51-200</t>
+          <t>11-50</t>
         </is>
       </c>
       <c r="I70" s="8" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>Tokyo, Japan</t>
         </is>
       </c>
       <c r="J70" s="8" t="inlineStr">
@@ -6469,7 +6465,7 @@
       <c r="M70" s="8" t="inlineStr"/>
       <c r="N70" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/liyashusterbier</t>
+          <t>https://www.linkedin.com/in/haruumi-shiode-ab17a83</t>
         </is>
       </c>
       <c r="O70" s="9" t="inlineStr"/>
@@ -6481,11 +6477,11 @@
       <c r="Q70" s="8" t="inlineStr"/>
       <c r="R70" s="8" t="inlineStr"/>
       <c r="S70" s="8" t="n">
-        <v>6557</v>
+        <v>3368</v>
       </c>
       <c r="T70" s="8" t="inlineStr">
         <is>
-          <t>6450</t>
+          <t>7371</t>
         </is>
       </c>
       <c r="U70" s="8" t="inlineStr">
@@ -6512,22 +6508,22 @@
       </c>
       <c r="D71" s="8" t="inlineStr">
         <is>
-          <t>Moms First (formerly Marshall Plan for Moms)</t>
+          <t>Nevis Capital</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t>Reshma Saujani</t>
+          <t>Colin Fraser</t>
         </is>
       </c>
       <c r="F71" s="8" t="inlineStr">
         <is>
-          <t>Founder and CEO</t>
+          <t>Co-Founder and Partner</t>
         </is>
       </c>
       <c r="G71" s="8" t="inlineStr">
         <is>
-          <t>Nonprofit</t>
+          <t>Private Equity</t>
         </is>
       </c>
       <c r="H71" s="8" t="inlineStr">
@@ -6537,7 +6533,7 @@
       </c>
       <c r="I71" s="8" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Nevis</t>
         </is>
       </c>
       <c r="J71" s="8" t="inlineStr">
@@ -6550,13 +6546,13 @@
       </c>
       <c r="L71" s="9" t="inlineStr">
         <is>
-          <t>David Yang</t>
+          <t>Joanna Patterson</t>
         </is>
       </c>
       <c r="M71" s="8" t="inlineStr"/>
       <c r="N71" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/reshma-saujani</t>
+          <t>https://www.linkedin.com/in/colinjfraser</t>
         </is>
       </c>
       <c r="O71" s="9" t="inlineStr"/>
@@ -6568,11 +6564,11 @@
       <c r="Q71" s="8" t="inlineStr"/>
       <c r="R71" s="8" t="inlineStr"/>
       <c r="S71" s="8" t="n">
-        <v>2342</v>
+        <v>9419</v>
       </c>
       <c r="T71" s="8" t="inlineStr">
         <is>
-          <t>7491</t>
+          <t>7377</t>
         </is>
       </c>
       <c r="U71" s="8" t="inlineStr">
@@ -6599,12 +6595,12 @@
       </c>
       <c r="D72" s="8" t="inlineStr">
         <is>
-          <t>Nature Inc. (Nature Remo)</t>
+          <t>OneGoal Prep</t>
         </is>
       </c>
       <c r="E72" s="8" t="inlineStr">
         <is>
-          <t>Haruumi Shiode</t>
+          <t>John Murphy</t>
         </is>
       </c>
       <c r="F72" s="8" t="inlineStr">
@@ -6614,7 +6610,7 @@
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
@@ -6624,7 +6620,7 @@
       </c>
       <c r="I72" s="8" t="inlineStr">
         <is>
-          <t>Tokyo, Japan</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="J72" s="8" t="inlineStr">
@@ -6643,7 +6639,7 @@
       <c r="M72" s="8" t="inlineStr"/>
       <c r="N72" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/haruumi-shiode-ab17a83</t>
+          <t>https://www.linkedin.com/in/johnmurphyaxiom</t>
         </is>
       </c>
       <c r="O72" s="9" t="inlineStr"/>
@@ -6655,11 +6651,11 @@
       <c r="Q72" s="8" t="inlineStr"/>
       <c r="R72" s="8" t="inlineStr"/>
       <c r="S72" s="8" t="n">
-        <v>3368</v>
+        <v>11583</v>
       </c>
       <c r="T72" s="8" t="inlineStr">
         <is>
-          <t>7371</t>
+          <t>8260</t>
         </is>
       </c>
       <c r="U72" s="8" t="inlineStr">
@@ -6686,32 +6682,32 @@
       </c>
       <c r="D73" s="8" t="inlineStr">
         <is>
-          <t>Nevis Capital</t>
+          <t>Panax</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t>Colin Fraser</t>
+          <t>Noam Mills</t>
         </is>
       </c>
       <c r="F73" s="8" t="inlineStr">
         <is>
-          <t>Co-Founder and Partner</t>
+          <t>Co-Founder &amp; CEO</t>
         </is>
       </c>
       <c r="G73" s="8" t="inlineStr">
         <is>
-          <t>Private Equity</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="H73" s="8" t="inlineStr">
         <is>
-          <t>11-50</t>
+          <t>1001-5000</t>
         </is>
       </c>
       <c r="I73" s="8" t="inlineStr">
         <is>
-          <t>Nevis</t>
+          <t>Seoul, South Korea</t>
         </is>
       </c>
       <c r="J73" s="8" t="inlineStr">
@@ -6730,7 +6726,7 @@
       <c r="M73" s="8" t="inlineStr"/>
       <c r="N73" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/colinjfraser</t>
+          <t>https://www.linkedin.com/in/noammills</t>
         </is>
       </c>
       <c r="O73" s="9" t="inlineStr"/>
@@ -6742,11 +6738,11 @@
       <c r="Q73" s="8" t="inlineStr"/>
       <c r="R73" s="8" t="inlineStr"/>
       <c r="S73" s="8" t="n">
-        <v>9419</v>
+        <v>1105</v>
       </c>
       <c r="T73" s="8" t="inlineStr">
         <is>
-          <t>7377</t>
+          <t>7004</t>
         </is>
       </c>
       <c r="U73" s="8" t="inlineStr">
@@ -6773,32 +6769,32 @@
       </c>
       <c r="D74" s="8" t="inlineStr">
         <is>
-          <t>OneGoal Prep</t>
+          <t>Passage Health</t>
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr">
         <is>
-          <t>John Murphy</t>
+          <t>Bill White</t>
         </is>
       </c>
       <c r="F74" s="8" t="inlineStr">
         <is>
-          <t>Founder</t>
+          <t>Co-Founder and CEO</t>
         </is>
       </c>
       <c r="G74" s="8" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr">
         <is>
-          <t>11-50</t>
+          <t>51-200</t>
         </is>
       </c>
       <c r="I74" s="8" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Indianapolis, IN</t>
         </is>
       </c>
       <c r="J74" s="8" t="inlineStr">
@@ -6817,7 +6813,7 @@
       <c r="M74" s="8" t="inlineStr"/>
       <c r="N74" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/johnmurphyaxiom</t>
+          <t>https://www.linkedin.com/in/bill-white-6aa2a520</t>
         </is>
       </c>
       <c r="O74" s="9" t="inlineStr"/>
@@ -6829,11 +6825,11 @@
       <c r="Q74" s="8" t="inlineStr"/>
       <c r="R74" s="8" t="inlineStr"/>
       <c r="S74" s="8" t="n">
-        <v>11583</v>
+        <v>8647</v>
       </c>
       <c r="T74" s="8" t="inlineStr">
         <is>
-          <t>8260</t>
+          <t>7059</t>
         </is>
       </c>
       <c r="U74" s="8" t="inlineStr">
@@ -6860,32 +6856,32 @@
       </c>
       <c r="D75" s="8" t="inlineStr">
         <is>
-          <t>Panax</t>
+          <t>Putnam Foundation</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
         <is>
-          <t>Noam Mills</t>
+          <t>Jessica Lawrence Quinn, SPHR, CFRE</t>
         </is>
       </c>
       <c r="F75" s="8" t="inlineStr">
         <is>
-          <t>Co-Founder &amp; CEO</t>
+          <t>Chief Executive Officer</t>
         </is>
       </c>
       <c r="G75" s="8" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Nonprofit</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr">
         <is>
-          <t>1001-5000</t>
+          <t>51-200</t>
         </is>
       </c>
       <c r="I75" s="8" t="inlineStr">
         <is>
-          <t>Seoul, South Korea</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="J75" s="8" t="inlineStr">
@@ -6898,13 +6894,13 @@
       </c>
       <c r="L75" s="9" t="inlineStr">
         <is>
-          <t>Joanna Patterson</t>
+          <t>David Yang</t>
         </is>
       </c>
       <c r="M75" s="8" t="inlineStr"/>
       <c r="N75" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/noammills</t>
+          <t>https://www.linkedin.com/in/jessicalawrencequinn</t>
         </is>
       </c>
       <c r="O75" s="9" t="inlineStr"/>
@@ -6916,11 +6912,11 @@
       <c r="Q75" s="8" t="inlineStr"/>
       <c r="R75" s="8" t="inlineStr"/>
       <c r="S75" s="8" t="n">
-        <v>1105</v>
+        <v>7111</v>
       </c>
       <c r="T75" s="8" t="inlineStr">
         <is>
-          <t>7004</t>
+          <t>7809</t>
         </is>
       </c>
       <c r="U75" s="8" t="inlineStr">
@@ -6947,22 +6943,22 @@
       </c>
       <c r="D76" s="8" t="inlineStr">
         <is>
-          <t>Passage Health</t>
+          <t>Quidnet Energy</t>
         </is>
       </c>
       <c r="E76" s="8" t="inlineStr">
         <is>
-          <t>Bill White</t>
+          <t>Joe Zhou</t>
         </is>
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
-          <t>Co-Founder and CEO</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="G76" s="8" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="H76" s="8" t="inlineStr">
@@ -6972,7 +6968,7 @@
       </c>
       <c r="I76" s="8" t="inlineStr">
         <is>
-          <t>Indianapolis, IN</t>
+          <t>Arlington, MA</t>
         </is>
       </c>
       <c r="J76" s="8" t="inlineStr">
@@ -6991,7 +6987,7 @@
       <c r="M76" s="8" t="inlineStr"/>
       <c r="N76" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/bill-white-6aa2a520</t>
+          <t>https://www.linkedin.com/in/jdzhou</t>
         </is>
       </c>
       <c r="O76" s="9" t="inlineStr"/>
@@ -7003,11 +6999,11 @@
       <c r="Q76" s="8" t="inlineStr"/>
       <c r="R76" s="8" t="inlineStr"/>
       <c r="S76" s="8" t="n">
-        <v>8647</v>
+        <v>5211</v>
       </c>
       <c r="T76" s="8" t="inlineStr">
         <is>
-          <t>7059</t>
+          <t>7813</t>
         </is>
       </c>
       <c r="U76" s="8" t="inlineStr">
@@ -7034,32 +7030,32 @@
       </c>
       <c r="D77" s="8" t="inlineStr">
         <is>
-          <t>Putnam Foundation</t>
+          <t>re/village</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
         <is>
-          <t>Jessica Lawrence Quinn, SPHR, CFRE</t>
+          <t>Matt Jorgensen</t>
         </is>
       </c>
       <c r="F77" s="8" t="inlineStr">
         <is>
-          <t>Chief Executive Officer</t>
+          <t>Co-Founder</t>
         </is>
       </c>
       <c r="G77" s="8" t="inlineStr">
         <is>
-          <t>Nonprofit</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="H77" s="8" t="inlineStr">
         <is>
-          <t>51-200</t>
+          <t>11-50</t>
         </is>
       </c>
       <c r="I77" s="8" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Brooklyn, NY</t>
         </is>
       </c>
       <c r="J77" s="8" t="inlineStr">
@@ -7072,13 +7068,13 @@
       </c>
       <c r="L77" s="9" t="inlineStr">
         <is>
-          <t>David Yang</t>
+          <t>Joanna Patterson</t>
         </is>
       </c>
       <c r="M77" s="8" t="inlineStr"/>
       <c r="N77" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/jessicalawrencequinn</t>
+          <t>https://www.linkedin.com/in/mattjorgensen1</t>
         </is>
       </c>
       <c r="O77" s="9" t="inlineStr"/>
@@ -7090,11 +7086,11 @@
       <c r="Q77" s="8" t="inlineStr"/>
       <c r="R77" s="8" t="inlineStr"/>
       <c r="S77" s="8" t="n">
-        <v>7111</v>
+        <v>11929</v>
       </c>
       <c r="T77" s="8" t="inlineStr">
         <is>
-          <t>7809</t>
+          <t>7609</t>
         </is>
       </c>
       <c r="U77" s="8" t="inlineStr">
@@ -7121,32 +7117,32 @@
       </c>
       <c r="D78" s="8" t="inlineStr">
         <is>
-          <t>Quidnet Energy</t>
+          <t>Sespe Health Holdings</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
         <is>
-          <t>Joe Zhou</t>
+          <t>Sander Duncan</t>
         </is>
       </c>
       <c r="F78" s="8" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Founder and CEO</t>
         </is>
       </c>
       <c r="G78" s="8" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="H78" s="8" t="inlineStr">
         <is>
-          <t>51-200</t>
+          <t>1001-5000</t>
         </is>
       </c>
       <c r="I78" s="8" t="inlineStr">
         <is>
-          <t>Arlington, MA</t>
+          <t>Ojai, CA</t>
         </is>
       </c>
       <c r="J78" s="8" t="inlineStr">
@@ -7165,7 +7161,7 @@
       <c r="M78" s="8" t="inlineStr"/>
       <c r="N78" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/jdzhou</t>
+          <t>https://www.linkedin.com/in/sanderduncan</t>
         </is>
       </c>
       <c r="O78" s="9" t="inlineStr"/>
@@ -7177,11 +7173,11 @@
       <c r="Q78" s="8" t="inlineStr"/>
       <c r="R78" s="8" t="inlineStr"/>
       <c r="S78" s="8" t="n">
-        <v>5211</v>
+        <v>10064</v>
       </c>
       <c r="T78" s="8" t="inlineStr">
         <is>
-          <t>7813</t>
+          <t>8747</t>
         </is>
       </c>
       <c r="U78" s="8" t="inlineStr">
@@ -7208,17 +7204,17 @@
       </c>
       <c r="D79" s="8" t="inlineStr">
         <is>
-          <t>re/village</t>
+          <t>Shiru</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
         <is>
-          <t>Matt Jorgensen</t>
+          <t>Jasmin Hume</t>
         </is>
       </c>
       <c r="F79" s="8" t="inlineStr">
         <is>
-          <t>Co-Founder</t>
+          <t>Founder and CEO</t>
         </is>
       </c>
       <c r="G79" s="8" t="inlineStr">
@@ -7233,7 +7229,7 @@
       </c>
       <c r="I79" s="8" t="inlineStr">
         <is>
-          <t>Brooklyn, NY</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="J79" s="8" t="inlineStr">
@@ -7246,13 +7242,13 @@
       </c>
       <c r="L79" s="9" t="inlineStr">
         <is>
-          <t>Joanna Patterson</t>
+          <t>David Yang</t>
         </is>
       </c>
       <c r="M79" s="8" t="inlineStr"/>
       <c r="N79" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mattjorgensen1</t>
+          <t>https://www.linkedin.com/in/jasminhume</t>
         </is>
       </c>
       <c r="O79" s="9" t="inlineStr"/>
@@ -7264,11 +7260,11 @@
       <c r="Q79" s="8" t="inlineStr"/>
       <c r="R79" s="8" t="inlineStr"/>
       <c r="S79" s="8" t="n">
-        <v>11929</v>
+        <v>6784</v>
       </c>
       <c r="T79" s="8" t="inlineStr">
         <is>
-          <t>7609</t>
+          <t>8801</t>
         </is>
       </c>
       <c r="U79" s="8" t="inlineStr">
@@ -7295,32 +7291,32 @@
       </c>
       <c r="D80" s="8" t="inlineStr">
         <is>
-          <t>Sespe Health Holdings</t>
+          <t>Showpad</t>
         </is>
       </c>
       <c r="E80" s="8" t="inlineStr">
         <is>
-          <t>Sander Duncan</t>
+          <t>Hendrik Isebaert</t>
         </is>
       </c>
       <c r="F80" s="8" t="inlineStr">
         <is>
-          <t>Founder and CEO</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="G80" s="8" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="H80" s="8" t="inlineStr">
         <is>
-          <t>1001-5000</t>
+          <t>201-1000</t>
         </is>
       </c>
       <c r="I80" s="8" t="inlineStr">
         <is>
-          <t>Ojai, CA</t>
+          <t>Ghent, Belgium</t>
         </is>
       </c>
       <c r="J80" s="8" t="inlineStr">
@@ -7339,7 +7335,7 @@
       <c r="M80" s="8" t="inlineStr"/>
       <c r="N80" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/sanderduncan</t>
+          <t>https://www.linkedin.com/in/hendrikisebaert</t>
         </is>
       </c>
       <c r="O80" s="9" t="inlineStr"/>
@@ -7351,11 +7347,11 @@
       <c r="Q80" s="8" t="inlineStr"/>
       <c r="R80" s="8" t="inlineStr"/>
       <c r="S80" s="8" t="n">
-        <v>10064</v>
+        <v>9408</v>
       </c>
       <c r="T80" s="8" t="inlineStr">
         <is>
-          <t>8747</t>
+          <t>8901</t>
         </is>
       </c>
       <c r="U80" s="8" t="inlineStr">
@@ -7382,22 +7378,22 @@
       </c>
       <c r="D81" s="8" t="inlineStr">
         <is>
-          <t>Shiru</t>
+          <t>Underscore VC</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr">
         <is>
-          <t>Jasmin Hume</t>
+          <t>Richard Dulude</t>
         </is>
       </c>
       <c r="F81" s="8" t="inlineStr">
         <is>
-          <t>Founder and CEO</t>
+          <t>Co-Founder &amp; General Partner</t>
         </is>
       </c>
       <c r="G81" s="8" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="H81" s="8" t="inlineStr">
@@ -7420,13 +7416,13 @@
       </c>
       <c r="L81" s="9" t="inlineStr">
         <is>
-          <t>David Yang</t>
+          <t>Joanna Patterson</t>
         </is>
       </c>
       <c r="M81" s="8" t="inlineStr"/>
       <c r="N81" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/jasminhume</t>
+          <t>https://www.linkedin.com/in/dulude</t>
         </is>
       </c>
       <c r="O81" s="9" t="inlineStr"/>
@@ -7438,11 +7434,11 @@
       <c r="Q81" s="8" t="inlineStr"/>
       <c r="R81" s="8" t="inlineStr"/>
       <c r="S81" s="8" t="n">
-        <v>6784</v>
+        <v>9337</v>
       </c>
       <c r="T81" s="8" t="inlineStr">
         <is>
-          <t>8801</t>
+          <t>9802</t>
         </is>
       </c>
       <c r="U81" s="8" t="inlineStr">
@@ -7451,182 +7447,8 @@
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="8" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="B82" s="8" t="inlineStr">
-        <is>
-          <t>Unassigned</t>
-        </is>
-      </c>
-      <c r="C82" s="8" t="inlineStr">
-        <is>
-          <t>No — wrong size or geo</t>
-        </is>
-      </c>
-      <c r="D82" s="8" t="inlineStr">
-        <is>
-          <t>Showpad</t>
-        </is>
-      </c>
-      <c r="E82" s="8" t="inlineStr">
-        <is>
-          <t>Hendrik Isebaert</t>
-        </is>
-      </c>
-      <c r="F82" s="8" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="G82" s="8" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="H82" s="8" t="inlineStr">
-        <is>
-          <t>201-1000</t>
-        </is>
-      </c>
-      <c r="I82" s="8" t="inlineStr">
-        <is>
-          <t>Ghent, Belgium</t>
-        </is>
-      </c>
-      <c r="J82" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K82" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L82" s="9" t="inlineStr">
-        <is>
-          <t>Joanna Patterson</t>
-        </is>
-      </c>
-      <c r="M82" s="8" t="inlineStr"/>
-      <c r="N82" s="8" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/hendrikisebaert</t>
-        </is>
-      </c>
-      <c r="O82" s="9" t="inlineStr"/>
-      <c r="P82" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="Q82" s="8" t="inlineStr"/>
-      <c r="R82" s="8" t="inlineStr"/>
-      <c r="S82" s="8" t="n">
-        <v>9408</v>
-      </c>
-      <c r="T82" s="8" t="inlineStr">
-        <is>
-          <t>8901</t>
-        </is>
-      </c>
-      <c r="U82" s="8" t="inlineStr">
-        <is>
-          <t>Operation 35 — LT (Joanna / Dave)</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="8" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="B83" s="8" t="inlineStr">
-        <is>
-          <t>Unassigned</t>
-        </is>
-      </c>
-      <c r="C83" s="8" t="inlineStr">
-        <is>
-          <t>No — wrong size or geo</t>
-        </is>
-      </c>
-      <c r="D83" s="8" t="inlineStr">
-        <is>
-          <t>Underscore VC</t>
-        </is>
-      </c>
-      <c r="E83" s="8" t="inlineStr">
-        <is>
-          <t>Richard Dulude</t>
-        </is>
-      </c>
-      <c r="F83" s="8" t="inlineStr">
-        <is>
-          <t>Co-Founder &amp; General Partner</t>
-        </is>
-      </c>
-      <c r="G83" s="8" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="H83" s="8" t="inlineStr">
-        <is>
-          <t>11-50</t>
-        </is>
-      </c>
-      <c r="I83" s="8" t="inlineStr">
-        <is>
-          <t>San Francisco, CA</t>
-        </is>
-      </c>
-      <c r="J83" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K83" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L83" s="9" t="inlineStr">
-        <is>
-          <t>Joanna Patterson</t>
-        </is>
-      </c>
-      <c r="M83" s="8" t="inlineStr"/>
-      <c r="N83" s="8" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/dulude</t>
-        </is>
-      </c>
-      <c r="O83" s="9" t="inlineStr"/>
-      <c r="P83" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="Q83" s="8" t="inlineStr"/>
-      <c r="R83" s="8" t="inlineStr"/>
-      <c r="S83" s="8" t="n">
-        <v>9337</v>
-      </c>
-      <c r="T83" s="8" t="inlineStr">
-        <is>
-          <t>9802</t>
-        </is>
-      </c>
-      <c r="U83" s="8" t="inlineStr">
-        <is>
-          <t>Operation 35 — LT (Joanna / Dave)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:U83"/>
+  <autoFilter ref="A1:U81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7637,7 +7459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -7676,7 +7498,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>82 leadership-team contacts, Nick Simmons' input EXCLUDED, in the same column layout as the</t>
+          <t>80 leadership-team contacts, Nick Simmons' input EXCLUDED, in the same column layout as the</t>
         </is>
       </c>
     </row>
@@ -7728,35 +7550,35 @@
       <c r="A11" s="11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>So the base of this file is operation_35_lt in full.</t>
+          <t>This file is operation_35_lt in full and NOTHING else - not one contact from operation_35_lt_nick.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>The Nick list is captured separately, so no carve-ins or exceptions were made here.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr"/>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Two contacts sit on Nick's list but were rated ONLY by Joanna or Dave, with no Nick input at all, so they are included:</t>
-        </is>
-      </c>
+      <c r="B13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr"/>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Jen Hensley (Con Edison) - rated by David Yang</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr"/>
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Sophia Schneider (Uniswap Labs) - rated by Joanna Patterson, Stefano Barros, Victoria Mayo</t>
+          <t>No contact from operation_35_lt_nick appears here, and no row carries a Nick Simmons rating.</t>
         </is>
       </c>
     </row>
@@ -7764,7 +7586,7 @@
       <c r="A16" s="11" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>They are marked in the 'LT tag source' column as 'LT_Nick list, but rated only by Joanna/Dave' - filter that column to drop them.</t>
+          <t>Raters present: Joanna Patterson (50), David Yang (30), Victoria Mayo (1 - a co-rater on one of Joanna's contacts).</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7594,7 @@
       <c r="A17" s="11" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Two other Nick-list contacts rated by Joanna (annie rittgers, Joey Mejias) were EXCLUDED because Nick also rated them.</t>
+          <t>Every contact has at least one recorded rating; the 48 vote-less contacts were all on Nick's list and are gone.</t>
         </is>
       </c>
     </row>
@@ -7783,12 +7605,12 @@
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>CRITERIA FIT?</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>No row in this file carries a Nick Simmons rating. Raters present: Joanna Patterson (51), David Yang (31),</t>
+          <t>Yes = company HQ in NY/NJ/CT AND size bucket 51-200 or 201-1000. 15 contacts qualify.</t>
         </is>
       </c>
     </row>
@@ -7796,7 +7618,7 @@
       <c r="A20" s="11" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Victoria Mayo (2), Stefano Barros (1). Every contact has at least one recorded rating - the 48 unrated contacts</t>
+          <t>No - wrong size or geo: 39.</t>
         </is>
       </c>
     </row>
@@ -7804,47 +7626,43 @@
       <c r="A21" s="11" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
-          <t>in the previous version were all on Nick's list and are now gone.</t>
+          <t>Unknown - company not enriched: 26 (company record has no HQ or no size bucket).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr"/>
-      <c r="B22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Unknown - no company linked: 0 (contact has no company_id at all).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t>CRITERIA FIT?</t>
-        </is>
-      </c>
+      <c r="A23" s="11" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Yes = company HQ in NY/NJ/CT AND size bucket 51-200 or 201-1000. 16 contacts qualify.</t>
+          <t>Unknown rows are kept, not dropped - the same treatment as the Staff tab.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr"/>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>No - wrong size or geo: 40.</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="inlineStr"/>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Unknown - company not enriched: 26 (company record has no HQ or no size bucket).</t>
-        </is>
-      </c>
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>!! PRIORITY IS A SUGGESTION !!</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Unknown - no company linked: 0 (contact has no company_id at all).</t>
+          <t>Priority in your Staff tab is assigned by hand and follows no rule I can reproduce (some P1 rows are</t>
         </is>
       </c>
     </row>
@@ -7852,27 +7670,31 @@
       <c r="A27" s="12" t="inlineStr"/>
       <c r="B27" s="13" t="inlineStr">
         <is>
-          <t>Unknown rows are kept, not dropped - the same treatment as the Staff tab.</t>
+          <t>'No - wrong size or geo', some P2 rows fit the criteria), so I did NOT try to reverse-engineer it.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr"/>
-      <c r="B28" s="13" t="inlineStr"/>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>The Priority column here is a computed STARTING POINT using this explicit rule - overwrite it freely:</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="inlineStr">
-        <is>
-          <t>!! PRIORITY IS A SUGGESTION !!</t>
-        </is>
-      </c>
-      <c r="B29" s="13" t="inlineStr"/>
+      <c r="A29" s="12" t="inlineStr"/>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   P1 = fits criteria AND hiring fit = yes   (7 contacts)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="12" t="inlineStr"/>
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>Priority in your Staff tab is assigned by hand and follows no rule I can reproduce (some P1 rows are</t>
+          <t xml:space="preserve">   P2 = fits criteria AND hiring fit = no    (8 contacts)</t>
         </is>
       </c>
     </row>
@@ -7880,7 +7702,7 @@
       <c r="A31" s="12" t="inlineStr"/>
       <c r="B31" s="13" t="inlineStr">
         <is>
-          <t>'No - wrong size or geo', some P2 rows fit the criteria), so I did NOT try to reverse-engineer it.</t>
+          <t xml:space="preserve">   P3 = criteria fit unknown                 (26 contacts)</t>
         </is>
       </c>
     </row>
@@ -7888,79 +7710,47 @@
       <c r="A32" s="12" t="inlineStr"/>
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>The Priority column here is a computed STARTING POINT using this explicit rule - overwrite it freely:</t>
+          <t xml:space="preserve">   P4 = does not fit on size or geography    (39 contacts)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="12" t="inlineStr"/>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   P1 = fits criteria AND hiring fit = yes   (7 contacts)</t>
-        </is>
-      </c>
+      <c r="B33" s="13" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="inlineStr"/>
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>ACCT. OWNER</t>
+        </is>
+      </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">   P2 = fits criteria AND hiring fit = no    (9 contacts)</t>
+          <t>Derived from contacts.owner_email; contacts without one show 'Unassigned' for you to fill in.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr"/>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   P3 = criteria fit unknown                 (26 contacts)</t>
-        </is>
-      </c>
+      <c r="B35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="11" t="inlineStr"/>
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>NOT INCLUDED</t>
+        </is>
+      </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">   P4 = does not fit on size or geography    (40 contacts)</t>
+          <t>operation_35_lt_nick (94 contacts) - excluded in full, captured elsewhere.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr"/>
-      <c r="B37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="11" t="inlineStr">
-        <is>
-          <t>ACCT. OWNER</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Derived from contacts.owner_email; contacts without one show 'Unassigned' for you to fill in.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="11" t="inlineStr"/>
-      <c r="B39" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="11" t="inlineStr">
-        <is>
-          <t>NOT INCLUDED</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>operation_35_pursuit (119 contacts, 17 of which fit the criteria) - a separate tag, not a leadership-team list.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="11" t="inlineStr"/>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>operation_35_lt_nick - excluded in full apart from the two contacts noted above.</t>
         </is>
       </c>
     </row>

</xml_diff>